<commit_message>
Update I&E sign handling and internal mappings
</commit_message>
<xml_diff>
--- a/src/lib/automation/ie/reference/To add I&E.xlsx
+++ b/src/lib/automation/ie/reference/To add I&E.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8fcd883c776305f1/Documentos/Veracity Automation/I^0E/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8fcd883c776305f1/Documentos/Keystone/keystone-os/src/lib/automation/ie/reference/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_20C4315295263003D1BD0F964BC8F3756E9CBE04" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{855D1640-E2EE-44B3-8B5E-F9AF9169E6DE}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="11_20C4315295263003D1BD0F964BC8F3756E9CBE04" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{46388C2D-BD95-4370-8A9C-4562E8A8A2D4}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -885,7 +885,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0_);\(0\)"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -911,13 +911,6 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
       <sz val="10"/>
       <color rgb="FFFF0000"/>
       <name val="Arial"/>
@@ -1022,55 +1015,53 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -1088,6 +1079,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1461,14 +1456,18 @@
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="12"/>
+      <c r="A11" s="12">
+        <v>41</v>
+      </c>
       <c r="B11" s="13" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="14"/>
-      <c r="B12" s="15" t="s">
+      <c r="A12" s="5">
+        <v>42</v>
+      </c>
+      <c r="B12" s="14" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1476,41 +1475,41 @@
       <c r="A13" s="5">
         <v>110</v>
       </c>
-      <c r="B13" s="16" t="s">
+      <c r="B13" s="14" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="17">
+      <c r="A14" s="15">
         <v>110</v>
       </c>
-      <c r="B14" s="18" t="s">
+      <c r="B14" s="16" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="5"/>
-      <c r="B15" s="16" t="s">
+      <c r="B15" s="14" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="17"/>
-      <c r="B16" s="19" t="s">
+      <c r="A16" s="15"/>
+      <c r="B16" s="17" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="20"/>
-      <c r="B17" s="16" t="s">
+      <c r="A17" s="18"/>
+      <c r="B17" s="14" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="17">
+      <c r="A18" s="15">
         <v>160</v>
       </c>
-      <c r="B18" s="19" t="s">
+      <c r="B18" s="17" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1518,986 +1517,986 @@
       <c r="A19" s="12">
         <v>160</v>
       </c>
-      <c r="B19" s="16" t="s">
+      <c r="B19" s="14" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="21">
+      <c r="A20" s="19">
         <v>160</v>
       </c>
-      <c r="B20" s="19" t="s">
+      <c r="B20" s="17" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="22">
+      <c r="A21" s="20">
         <v>160</v>
       </c>
-      <c r="B21" s="16" t="s">
+      <c r="B21" s="14" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="23">
+      <c r="A22" s="21">
         <v>160</v>
       </c>
-      <c r="B22" s="19" t="s">
+      <c r="B22" s="17" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="24">
+      <c r="A23" s="22">
         <v>160</v>
       </c>
-      <c r="B23" s="16" t="s">
+      <c r="B23" s="14" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" s="25">
+      <c r="A24" s="23">
         <v>160</v>
       </c>
-      <c r="B24" s="19" t="s">
+      <c r="B24" s="17" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" s="24">
+      <c r="A25" s="22">
         <v>160</v>
       </c>
-      <c r="B25" s="16" t="s">
+      <c r="B25" s="14" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" s="25">
+      <c r="A26" s="23">
         <v>160</v>
       </c>
-      <c r="B26" s="19" t="s">
+      <c r="B26" s="17" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" s="24">
+      <c r="A27" s="22">
         <v>160</v>
       </c>
-      <c r="B27" s="16" t="s">
+      <c r="B27" s="14" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" s="25">
+      <c r="A28" s="23">
         <v>160</v>
       </c>
-      <c r="B28" s="19" t="s">
+      <c r="B28" s="17" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" s="24">
+      <c r="A29" s="22">
         <v>160</v>
       </c>
-      <c r="B29" s="16" t="s">
+      <c r="B29" s="14" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30" s="25">
+      <c r="A30" s="23">
         <v>160</v>
       </c>
-      <c r="B30" s="19" t="s">
+      <c r="B30" s="17" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" s="24">
+      <c r="A31" s="22">
         <v>140</v>
       </c>
-      <c r="B31" s="16" t="s">
+      <c r="B31" s="14" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32" s="25">
+      <c r="A32" s="23">
         <v>160</v>
       </c>
-      <c r="B32" s="19" t="s">
+      <c r="B32" s="17" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" s="24">
+      <c r="A33" s="22">
         <v>160</v>
       </c>
-      <c r="B33" s="16" t="s">
+      <c r="B33" s="14" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" s="25">
+      <c r="A34" s="23">
         <v>160</v>
       </c>
-      <c r="B34" s="19" t="s">
+      <c r="B34" s="17" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A35" s="24">
+      <c r="A35" s="22">
         <v>103</v>
       </c>
-      <c r="B35" s="16" t="s">
+      <c r="B35" s="14" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A36" s="25">
+      <c r="A36" s="23">
         <v>103</v>
       </c>
-      <c r="B36" s="19" t="s">
+      <c r="B36" s="17" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A37" s="24"/>
-      <c r="B37" s="16" t="s">
+      <c r="A37" s="22"/>
+      <c r="B37" s="14" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38" s="26"/>
-      <c r="B38" s="18" t="s">
+      <c r="A38" s="24"/>
+      <c r="B38" s="16" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A39" s="24"/>
-      <c r="B39" s="16" t="s">
+      <c r="A39" s="22"/>
+      <c r="B39" s="14" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A40" s="25"/>
-      <c r="B40" s="18" t="s">
+      <c r="A40" s="23"/>
+      <c r="B40" s="16" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A41" s="24">
-        <v>41</v>
-      </c>
-      <c r="B41" s="16" t="s">
+      <c r="A41" s="22">
+        <v>41</v>
+      </c>
+      <c r="B41" s="14" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A42" s="25">
-        <v>41</v>
-      </c>
-      <c r="B42" s="18" t="s">
+      <c r="A42" s="23">
+        <v>41</v>
+      </c>
+      <c r="B42" s="16" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A43" s="24">
-        <v>41</v>
-      </c>
-      <c r="B43" s="16" t="s">
+      <c r="A43" s="22">
+        <v>41</v>
+      </c>
+      <c r="B43" s="14" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A44" s="25">
-        <v>41</v>
-      </c>
-      <c r="B44" s="19" t="s">
+      <c r="A44" s="23">
+        <v>41</v>
+      </c>
+      <c r="B44" s="17" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A45" s="27">
-        <v>41</v>
-      </c>
-      <c r="B45" s="16" t="s">
+      <c r="A45" s="25">
+        <v>41</v>
+      </c>
+      <c r="B45" s="14" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A46" s="26">
-        <v>41</v>
-      </c>
-      <c r="B46" s="19" t="s">
+      <c r="A46" s="24">
+        <v>41</v>
+      </c>
+      <c r="B46" s="17" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A47" s="27">
-        <v>41</v>
-      </c>
-      <c r="B47" s="16" t="s">
+      <c r="A47" s="25">
+        <v>41</v>
+      </c>
+      <c r="B47" s="14" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A48" s="25">
-        <v>41</v>
-      </c>
-      <c r="B48" s="19" t="s">
+      <c r="A48" s="23">
+        <v>41</v>
+      </c>
+      <c r="B48" s="17" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A49" s="24">
-        <v>41</v>
-      </c>
-      <c r="B49" s="16" t="s">
+      <c r="A49" s="22">
+        <v>41</v>
+      </c>
+      <c r="B49" s="14" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A50" s="26">
-        <v>41</v>
-      </c>
-      <c r="B50" s="19" t="s">
+      <c r="A50" s="24">
+        <v>41</v>
+      </c>
+      <c r="B50" s="17" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A51" s="24">
-        <v>41</v>
-      </c>
-      <c r="B51" s="16" t="s">
+      <c r="A51" s="22">
+        <v>41</v>
+      </c>
+      <c r="B51" s="14" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A52" s="25">
-        <v>41</v>
-      </c>
-      <c r="B52" s="19" t="s">
+      <c r="A52" s="23">
+        <v>41</v>
+      </c>
+      <c r="B52" s="17" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A53" s="24">
-        <v>41</v>
-      </c>
-      <c r="B53" s="16" t="s">
+      <c r="A53" s="22">
+        <v>41</v>
+      </c>
+      <c r="B53" s="14" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A54" s="25">
-        <v>41</v>
-      </c>
-      <c r="B54" s="19" t="s">
+      <c r="A54" s="23">
+        <v>41</v>
+      </c>
+      <c r="B54" s="17" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A55" s="24">
-        <v>41</v>
-      </c>
-      <c r="B55" s="16" t="s">
+      <c r="A55" s="22">
+        <v>41</v>
+      </c>
+      <c r="B55" s="14" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A56" s="25">
-        <v>41</v>
-      </c>
-      <c r="B56" s="19" t="s">
+      <c r="A56" s="23">
+        <v>41</v>
+      </c>
+      <c r="B56" s="17" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A57" s="24">
-        <v>41</v>
-      </c>
-      <c r="B57" s="16" t="s">
+      <c r="A57" s="22">
+        <v>41</v>
+      </c>
+      <c r="B57" s="14" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A58" s="25">
-        <v>41</v>
-      </c>
-      <c r="B58" s="19" t="s">
+      <c r="A58" s="23">
+        <v>41</v>
+      </c>
+      <c r="B58" s="17" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A59" s="24">
-        <v>41</v>
-      </c>
-      <c r="B59" s="16" t="s">
+      <c r="A59" s="22">
+        <v>41</v>
+      </c>
+      <c r="B59" s="14" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A60" s="25">
-        <v>41</v>
-      </c>
-      <c r="B60" s="19" t="s">
+      <c r="A60" s="23">
+        <v>41</v>
+      </c>
+      <c r="B60" s="17" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A61" s="24">
-        <v>41</v>
-      </c>
-      <c r="B61" s="16" t="s">
+      <c r="A61" s="22">
+        <v>41</v>
+      </c>
+      <c r="B61" s="14" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A62" s="25">
-        <v>41</v>
-      </c>
-      <c r="B62" s="19" t="s">
+      <c r="A62" s="23">
+        <v>41</v>
+      </c>
+      <c r="B62" s="17" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A63" s="24"/>
-      <c r="B63" s="16" t="s">
+      <c r="A63" s="22"/>
+      <c r="B63" s="14" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A64" s="25"/>
-      <c r="B64" s="19" t="s">
+      <c r="A64" s="23"/>
+      <c r="B64" s="17" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A65" s="24">
+      <c r="A65" s="22">
         <v>43</v>
       </c>
-      <c r="B65" s="16" t="s">
+      <c r="B65" s="14" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A66" s="25">
+      <c r="A66" s="23">
         <v>43</v>
       </c>
-      <c r="B66" s="18" t="s">
+      <c r="B66" s="16" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A67" s="24">
+      <c r="A67" s="22">
         <v>43</v>
       </c>
-      <c r="B67" s="16" t="s">
+      <c r="B67" s="14" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A68" s="25">
+      <c r="A68" s="23">
         <v>43</v>
       </c>
-      <c r="B68" s="18" t="s">
+      <c r="B68" s="16" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A69" s="24">
+      <c r="A69" s="22">
         <v>43</v>
       </c>
-      <c r="B69" s="16" t="s">
+      <c r="B69" s="14" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A70" s="25">
+      <c r="A70" s="23">
         <v>43</v>
       </c>
-      <c r="B70" s="18" t="s">
+      <c r="B70" s="16" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A71" s="24">
+      <c r="A71" s="22">
         <v>43</v>
       </c>
-      <c r="B71" s="16" t="s">
+      <c r="B71" s="14" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A72" s="25">
+      <c r="A72" s="23">
         <v>43</v>
       </c>
-      <c r="B72" s="18" t="s">
+      <c r="B72" s="16" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A73" s="24">
+      <c r="A73" s="22">
         <v>43</v>
       </c>
-      <c r="B73" s="16" t="s">
+      <c r="B73" s="14" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A74" s="25"/>
-      <c r="B74" s="18" t="s">
+      <c r="A74" s="23"/>
+      <c r="B74" s="16" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A75" s="24"/>
-      <c r="B75" s="16" t="s">
+      <c r="A75" s="22"/>
+      <c r="B75" s="14" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A76" s="25">
-        <v>11</v>
-      </c>
-      <c r="B76" s="19" t="s">
+      <c r="A76" s="23">
+        <v>11</v>
+      </c>
+      <c r="B76" s="17" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A77" s="24">
-        <v>11</v>
-      </c>
-      <c r="B77" s="16" t="s">
+      <c r="A77" s="22">
+        <v>11</v>
+      </c>
+      <c r="B77" s="14" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A78" s="25">
-        <v>11</v>
-      </c>
-      <c r="B78" s="19" t="s">
+      <c r="A78" s="23">
+        <v>11</v>
+      </c>
+      <c r="B78" s="17" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A79" s="24">
+      <c r="A79" s="22">
         <v>13</v>
       </c>
-      <c r="B79" s="16" t="s">
+      <c r="B79" s="14" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A80" s="25">
+      <c r="A80" s="23">
         <v>13</v>
       </c>
-      <c r="B80" s="19" t="s">
+      <c r="B80" s="17" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A81" s="24">
-        <v>11</v>
-      </c>
-      <c r="B81" s="16" t="s">
+      <c r="A81" s="22">
+        <v>11</v>
+      </c>
+      <c r="B81" s="14" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A82" s="25">
-        <v>11</v>
-      </c>
-      <c r="B82" s="19" t="s">
+      <c r="A82" s="23">
+        <v>11</v>
+      </c>
+      <c r="B82" s="17" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A83" s="24">
-        <v>11</v>
-      </c>
-      <c r="B83" s="16" t="s">
+      <c r="A83" s="22">
+        <v>11</v>
+      </c>
+      <c r="B83" s="14" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A84" s="25">
-        <v>11</v>
-      </c>
-      <c r="B84" s="19" t="s">
+      <c r="A84" s="23">
+        <v>11</v>
+      </c>
+      <c r="B84" s="17" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A85" s="24">
-        <v>11</v>
-      </c>
-      <c r="B85" s="16" t="s">
+      <c r="A85" s="22">
+        <v>11</v>
+      </c>
+      <c r="B85" s="14" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A86" s="25">
-        <v>11</v>
-      </c>
-      <c r="B86" s="19" t="s">
+      <c r="A86" s="23">
+        <v>11</v>
+      </c>
+      <c r="B86" s="17" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A87" s="24">
-        <v>11</v>
-      </c>
-      <c r="B87" s="16" t="s">
+      <c r="A87" s="22">
+        <v>11</v>
+      </c>
+      <c r="B87" s="14" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A88" s="25">
-        <v>11</v>
-      </c>
-      <c r="B88" s="19" t="s">
+      <c r="A88" s="23">
+        <v>11</v>
+      </c>
+      <c r="B88" s="17" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A89" s="24"/>
-      <c r="B89" s="16" t="s">
+      <c r="A89" s="22"/>
+      <c r="B89" s="14" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A90" s="25"/>
-      <c r="B90" s="19" t="s">
+      <c r="A90" s="23"/>
+      <c r="B90" s="17" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A91" s="24">
+      <c r="A91" s="22">
         <v>12</v>
       </c>
-      <c r="B91" s="16" t="s">
+      <c r="B91" s="14" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A92" s="25">
+      <c r="A92" s="23">
         <v>12</v>
       </c>
-      <c r="B92" s="19" t="s">
+      <c r="B92" s="17" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A93" s="24">
+      <c r="A93" s="22">
         <v>12</v>
       </c>
-      <c r="B93" s="28" t="s">
+      <c r="B93" s="26" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A94" s="25">
-        <v>11</v>
-      </c>
-      <c r="B94" s="18" t="s">
+      <c r="A94" s="23">
+        <v>11</v>
+      </c>
+      <c r="B94" s="16" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A95" s="24">
+      <c r="A95" s="22">
         <v>15</v>
       </c>
-      <c r="B95" s="16" t="s">
+      <c r="B95" s="14" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A96" s="25">
-        <v>11</v>
-      </c>
-      <c r="B96" s="18" t="s">
+      <c r="A96" s="23">
+        <v>11</v>
+      </c>
+      <c r="B96" s="16" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A97" s="24">
-        <v>11</v>
-      </c>
-      <c r="B97" s="16" t="s">
+      <c r="A97" s="22">
+        <v>11</v>
+      </c>
+      <c r="B97" s="14" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A98" s="25">
+      <c r="A98" s="23">
         <v>13</v>
       </c>
-      <c r="B98" s="18" t="s">
+      <c r="B98" s="16" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A99" s="24">
+      <c r="A99" s="22">
         <v>13</v>
       </c>
-      <c r="B99" s="16" t="s">
+      <c r="B99" s="14" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A100" s="25">
+      <c r="A100" s="23">
         <v>12</v>
       </c>
-      <c r="B100" s="18" t="s">
+      <c r="B100" s="16" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A101" s="24">
-        <v>11</v>
-      </c>
-      <c r="B101" s="28" t="s">
+      <c r="A101" s="22">
+        <v>11</v>
+      </c>
+      <c r="B101" s="26" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A102" s="25">
-        <v>11</v>
-      </c>
-      <c r="B102" s="19" t="s">
+      <c r="A102" s="23">
+        <v>11</v>
+      </c>
+      <c r="B102" s="17" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A103" s="24">
-        <v>11</v>
-      </c>
-      <c r="B103" s="28" t="s">
+      <c r="A103" s="22">
+        <v>11</v>
+      </c>
+      <c r="B103" s="26" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A104" s="26">
+      <c r="A104" s="24">
         <v>13</v>
       </c>
-      <c r="B104" s="19" t="s">
+      <c r="B104" s="17" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A105" s="24">
+      <c r="A105" s="22">
         <v>16</v>
       </c>
-      <c r="B105" s="16" t="s">
+      <c r="B105" s="14" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A106" s="25"/>
-      <c r="B106" s="19" t="s">
+      <c r="A106" s="23"/>
+      <c r="B106" s="17" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A107" s="24"/>
-      <c r="B107" s="16" t="s">
+      <c r="A107" s="22"/>
+      <c r="B107" s="14" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A108" s="25"/>
-      <c r="B108" s="19" t="s">
+      <c r="A108" s="23"/>
+      <c r="B108" s="17" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="109" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A109" s="24">
+      <c r="A109" s="22">
         <v>42</v>
       </c>
-      <c r="B109" s="16" t="s">
+      <c r="B109" s="14" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A110" s="25">
+      <c r="A110" s="23">
         <v>42</v>
       </c>
-      <c r="B110" s="19" t="s">
+      <c r="B110" s="17" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="111" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A111" s="24">
+      <c r="A111" s="22">
         <v>42</v>
       </c>
-      <c r="B111" s="28" t="s">
+      <c r="B111" s="26" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="112" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A112" s="25">
+      <c r="A112" s="23">
         <v>42</v>
       </c>
-      <c r="B112" s="19" t="s">
+      <c r="B112" s="17" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="113" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A113" s="24">
+      <c r="A113" s="22">
         <v>42</v>
       </c>
-      <c r="B113" s="28" t="s">
+      <c r="B113" s="26" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="114" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A114" s="25">
+      <c r="A114" s="23">
         <v>42</v>
       </c>
-      <c r="B114" s="19" t="s">
+      <c r="B114" s="17" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="115" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A115" s="24">
+      <c r="A115" s="22">
         <v>42</v>
       </c>
-      <c r="B115" s="28" t="s">
+      <c r="B115" s="26" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="116" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A116" s="25">
+      <c r="A116" s="23">
         <v>42</v>
       </c>
-      <c r="B116" s="19" t="s">
+      <c r="B116" s="17" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="117" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A117" s="24">
+      <c r="A117" s="22">
         <v>42</v>
       </c>
-      <c r="B117" s="28" t="s">
+      <c r="B117" s="26" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="118" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A118" s="25">
+      <c r="A118" s="23">
         <v>42</v>
       </c>
-      <c r="B118" s="19" t="s">
+      <c r="B118" s="17" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A119" s="24">
+      <c r="A119" s="22">
         <v>42</v>
       </c>
-      <c r="B119" s="16" t="s">
+      <c r="B119" s="14" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="120" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A120" s="25">
+      <c r="A120" s="23">
         <v>42</v>
       </c>
-      <c r="B120" s="29" t="s">
+      <c r="B120" s="27" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="121" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A121" s="24">
+      <c r="A121" s="22">
         <v>42</v>
       </c>
-      <c r="B121" s="16" t="s">
+      <c r="B121" s="14" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="122" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A122" s="25">
+      <c r="A122" s="23">
         <v>42</v>
       </c>
-      <c r="B122" s="19" t="s">
+      <c r="B122" s="17" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="123" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A123" s="24">
+      <c r="A123" s="22">
         <v>42</v>
       </c>
-      <c r="B123" s="16" t="s">
+      <c r="B123" s="14" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="124" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A124" s="25"/>
-      <c r="B124" s="19" t="s">
+      <c r="A124" s="23"/>
+      <c r="B124" s="17" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="125" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A125" s="24">
+      <c r="A125" s="22">
         <v>21</v>
       </c>
-      <c r="B125" s="16" t="s">
+      <c r="B125" s="14" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="126" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A126" s="25">
+      <c r="A126" s="23">
         <v>21</v>
       </c>
-      <c r="B126" s="19" t="s">
+      <c r="B126" s="17" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="127" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A127" s="24">
+      <c r="A127" s="22">
         <v>23</v>
       </c>
-      <c r="B127" s="16" t="s">
+      <c r="B127" s="14" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="128" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A128" s="25">
+      <c r="A128" s="23">
         <v>23</v>
       </c>
-      <c r="B128" s="19" t="s">
+      <c r="B128" s="17" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="129" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A129" s="24">
+      <c r="A129" s="22">
         <v>22</v>
       </c>
-      <c r="B129" s="16" t="s">
+      <c r="B129" s="14" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="130" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A130" s="25">
+      <c r="A130" s="23">
         <v>22</v>
       </c>
-      <c r="B130" s="19" t="s">
+      <c r="B130" s="17" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="131" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A131" s="27"/>
-      <c r="B131" s="16" t="s">
+      <c r="A131" s="25"/>
+      <c r="B131" s="14" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="132" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A132" s="25"/>
-      <c r="B132" s="19" t="s">
+      <c r="A132" s="23"/>
+      <c r="B132" s="17" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="133" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A133" s="24">
+      <c r="A133" s="22">
         <v>30</v>
       </c>
-      <c r="B133" s="16" t="s">
+      <c r="B133" s="14" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="134" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A134" s="25"/>
-      <c r="B134" s="19" t="s">
+      <c r="A134" s="23"/>
+      <c r="B134" s="17" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="135" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A135" s="22"/>
-      <c r="B135" s="16" t="s">
+      <c r="A135" s="20"/>
+      <c r="B135" s="14" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="136" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A136" s="23"/>
-      <c r="B136" s="19" t="s">
+      <c r="A136" s="21"/>
+      <c r="B136" s="17" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="137" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A137" s="24">
+      <c r="A137" s="22">
         <v>50</v>
       </c>
-      <c r="B137" s="16" t="s">
+      <c r="B137" s="14" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="138" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A138" s="25">
-        <v>41</v>
-      </c>
-      <c r="B138" s="19" t="s">
+      <c r="A138" s="23">
+        <v>41</v>
+      </c>
+      <c r="B138" s="17" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="139" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A139" s="24">
-        <v>41</v>
-      </c>
-      <c r="B139" s="16" t="s">
+      <c r="A139" s="22">
+        <v>41</v>
+      </c>
+      <c r="B139" s="14" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="140" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A140" s="25">
+      <c r="A140" s="23">
         <v>60</v>
       </c>
-      <c r="B140" s="19" t="s">
+      <c r="B140" s="17" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="141" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A141" s="24">
-        <v>41</v>
-      </c>
-      <c r="B141" s="16" t="s">
+      <c r="A141" s="22">
+        <v>41</v>
+      </c>
+      <c r="B141" s="14" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="142" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A142" s="25"/>
-      <c r="B142" s="19" t="s">
+      <c r="A142" s="23"/>
+      <c r="B142" s="17" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="143" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A143" s="24"/>
-      <c r="B143" s="16" t="s">
+      <c r="A143" s="22"/>
+      <c r="B143" s="14" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="144" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A144" s="26">
+      <c r="A144" s="24">
         <v>111</v>
       </c>
-      <c r="B144" s="19" t="s">
+      <c r="B144" s="17" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="145" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A145" s="24">
-        <v>41</v>
-      </c>
-      <c r="B145" s="16" t="s">
+      <c r="A145" s="22">
+        <v>41</v>
+      </c>
+      <c r="B145" s="14" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="146" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A146" s="25">
+      <c r="A146" s="23">
         <v>55</v>
       </c>
-      <c r="B146" s="19" t="s">
+      <c r="B146" s="17" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="147" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A147" s="30">
+      <c r="A147" s="28">
         <v>115</v>
       </c>
       <c r="B147" s="6" t="s">
@@ -2505,303 +2504,303 @@
       </c>
     </row>
     <row r="148" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A148" s="25">
+      <c r="A148" s="23">
         <v>142</v>
       </c>
-      <c r="B148" s="19" t="s">
+      <c r="B148" s="17" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="149" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A149" s="24">
+      <c r="A149" s="22">
         <v>142</v>
       </c>
-      <c r="B149" s="16" t="s">
+      <c r="B149" s="14" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="150" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A150" s="25">
+      <c r="A150" s="23">
         <v>160</v>
       </c>
-      <c r="B150" s="19" t="s">
+      <c r="B150" s="17" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="151" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A151" s="24">
-        <v>41</v>
-      </c>
-      <c r="B151" s="28" t="s">
+      <c r="A151" s="22">
+        <v>41</v>
+      </c>
+      <c r="B151" s="26" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="152" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A152" s="25">
-        <v>41</v>
-      </c>
-      <c r="B152" s="18" t="s">
+      <c r="A152" s="23">
+        <v>41</v>
+      </c>
+      <c r="B152" s="16" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="153" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A153" s="24">
+      <c r="A153" s="22">
         <v>24</v>
       </c>
-      <c r="B153" s="16" t="s">
+      <c r="B153" s="14" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="154" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A154" s="25">
-        <v>11</v>
-      </c>
-      <c r="B154" s="19" t="s">
+      <c r="A154" s="23">
+        <v>11</v>
+      </c>
+      <c r="B154" s="17" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="155" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A155" s="24">
-        <v>11</v>
-      </c>
-      <c r="B155" s="16" t="s">
+      <c r="A155" s="22">
+        <v>11</v>
+      </c>
+      <c r="B155" s="14" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="156" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A156" s="25">
-        <v>11</v>
-      </c>
-      <c r="B156" s="19" t="s">
+      <c r="A156" s="23">
+        <v>11</v>
+      </c>
+      <c r="B156" s="17" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="157" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A157" s="24">
-        <v>11</v>
-      </c>
-      <c r="B157" s="16" t="s">
+      <c r="A157" s="22">
+        <v>11</v>
+      </c>
+      <c r="B157" s="14" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="158" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A158" s="25">
-        <v>11</v>
-      </c>
-      <c r="B158" s="19" t="s">
+      <c r="A158" s="23">
+        <v>11</v>
+      </c>
+      <c r="B158" s="17" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="159" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A159" s="24">
-        <v>11</v>
-      </c>
-      <c r="B159" s="16" t="s">
+      <c r="A159" s="22">
+        <v>11</v>
+      </c>
+      <c r="B159" s="14" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="160" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A160" s="25">
-        <v>11</v>
-      </c>
-      <c r="B160" s="19" t="s">
+      <c r="A160" s="23">
+        <v>11</v>
+      </c>
+      <c r="B160" s="17" t="s">
         <v>157</v>
       </c>
     </row>
     <row r="161" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A161" s="24">
+      <c r="A161" s="22">
         <v>12</v>
       </c>
-      <c r="B161" s="16" t="s">
+      <c r="B161" s="14" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="162" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A162" s="25">
+      <c r="A162" s="23">
         <v>16</v>
       </c>
-      <c r="B162" s="18" t="s">
+      <c r="B162" s="16" t="s">
         <v>159</v>
       </c>
     </row>
     <row r="163" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A163" s="24">
-        <v>11</v>
-      </c>
-      <c r="B163" s="16" t="s">
+      <c r="A163" s="22">
+        <v>11</v>
+      </c>
+      <c r="B163" s="14" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="164" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A164" s="25"/>
-      <c r="B164" s="18" t="s">
+      <c r="A164" s="23"/>
+      <c r="B164" s="16" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="165" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A165" s="24"/>
-      <c r="B165" s="28" t="s">
+      <c r="A165" s="22"/>
+      <c r="B165" s="26" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="166" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A166" s="25"/>
-      <c r="B166" s="19" t="s">
+      <c r="A166" s="23"/>
+      <c r="B166" s="17" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="167" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A167" s="24"/>
-      <c r="B167" s="16" t="s">
+      <c r="A167" s="22"/>
+      <c r="B167" s="14" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="168" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A168" s="25">
-        <v>41</v>
-      </c>
-      <c r="B168" s="19" t="s">
+      <c r="A168" s="23">
+        <v>41</v>
+      </c>
+      <c r="B168" s="17" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="169" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A169" s="24">
-        <v>41</v>
-      </c>
-      <c r="B169" s="16" t="s">
+      <c r="A169" s="22">
+        <v>41</v>
+      </c>
+      <c r="B169" s="14" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="170" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A170" s="31">
+      <c r="A170" s="29">
         <v>121</v>
       </c>
-      <c r="B170" s="19" t="s">
+      <c r="B170" s="17" t="s">
         <v>166</v>
       </c>
     </row>
     <row r="171" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A171" s="30">
+      <c r="A171" s="28">
         <v>121</v>
       </c>
-      <c r="B171" s="16" t="s">
+      <c r="B171" s="14" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="172" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A172" s="25">
+      <c r="A172" s="23">
         <v>141</v>
       </c>
-      <c r="B172" s="19" t="s">
+      <c r="B172" s="17" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="173" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A173" s="24"/>
-      <c r="B173" s="16" t="s">
+      <c r="A173" s="22"/>
+      <c r="B173" s="14" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="174" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A174" s="25"/>
-      <c r="B174" s="18"/>
+      <c r="A174" s="23"/>
+      <c r="B174" s="16"/>
     </row>
     <row r="175" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A175" s="24">
-        <v>41</v>
-      </c>
-      <c r="B175" s="28" t="s">
+      <c r="A175" s="22">
+        <v>41</v>
+      </c>
+      <c r="B175" s="26" t="s">
         <v>169</v>
       </c>
     </row>
     <row r="176" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A176" s="25">
-        <v>41</v>
-      </c>
-      <c r="B176" s="18" t="s">
+      <c r="A176" s="23">
+        <v>41</v>
+      </c>
+      <c r="B176" s="16" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="177" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A177" s="24">
+      <c r="A177" s="22">
         <v>22</v>
       </c>
-      <c r="B177" s="16" t="s">
+      <c r="B177" s="14" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="178" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A178" s="25">
+      <c r="A178" s="23">
         <v>30</v>
       </c>
-      <c r="B178" s="19" t="s">
+      <c r="B178" s="17" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="179" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A179" s="24">
-        <v>41</v>
-      </c>
-      <c r="B179" s="32" t="str">
+      <c r="A179" s="22">
+        <v>41</v>
+      </c>
+      <c r="B179" s="30" t="str">
         <f>B12</f>
         <v>Employee Discounts</v>
       </c>
     </row>
     <row r="180" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A180" s="25">
+      <c r="A180" s="23">
         <v>42</v>
       </c>
-      <c r="B180" s="29" t="str">
+      <c r="B180" s="27" t="str">
         <f>B13</f>
         <v>Current Month Delinquency</v>
       </c>
     </row>
     <row r="181" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A181" s="24">
+      <c r="A181" s="22">
         <v>42</v>
       </c>
-      <c r="B181" s="16" t="s">
+      <c r="B181" s="14" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="182" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A182" s="25">
-        <v>11</v>
-      </c>
-      <c r="B182" s="19" t="s">
+      <c r="A182" s="23">
+        <v>11</v>
+      </c>
+      <c r="B182" s="17" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="183" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A183" s="24">
-        <v>11</v>
-      </c>
-      <c r="B183" s="16" t="s">
+      <c r="A183" s="22">
+        <v>11</v>
+      </c>
+      <c r="B183" s="14" t="s">
         <v>175</v>
       </c>
     </row>
     <row r="184" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A184" s="25">
+      <c r="A184" s="23">
         <v>55</v>
       </c>
-      <c r="B184" s="19" t="s">
+      <c r="B184" s="17" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="185" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A185" s="24">
-        <v>41</v>
-      </c>
-      <c r="B185" s="32" t="str">
+      <c r="A185" s="22">
+        <v>41</v>
+      </c>
+      <c r="B185" s="30" t="str">
         <f>B17</f>
         <v>Other Income</v>
       </c>
     </row>
     <row r="186" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A186" s="33">
+      <c r="A186" s="31">
         <v>42</v>
       </c>
-      <c r="B186" s="34" t="str">
+      <c r="B186" s="32" t="str">
         <f>B18</f>
         <v>Insufficient Notice</v>
       </c>

</xml_diff>

<commit_message>
Fix Employee Discounts internal mapping
</commit_message>
<xml_diff>
--- a/src/lib/automation/ie/reference/To add I&E.xlsx
+++ b/src/lib/automation/ie/reference/To add I&E.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8fcd883c776305f1/Documentos/Keystone/keystone-os/src/lib/automation/ie/reference/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="11_20C4315295263003D1BD0F964BC8F3756E9CBE04" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{46388C2D-BD95-4370-8A9C-4562E8A8A2D4}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="11_20C4315295263003D1BD0F964BC8F3756E9CBE04" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E4ACADDF-F71B-48EE-BD48-8714C68D5F2A}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1382,7 +1382,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:B291"/>
+  <dimension ref="A2:B290"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.28515625" customWidth="1"/>
@@ -2738,71 +2738,70 @@
       </c>
     </row>
     <row r="179" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A179" s="22">
-        <v>41</v>
-      </c>
-      <c r="B179" s="30" t="str">
-        <f>B12</f>
-        <v>Employee Discounts</v>
-      </c>
-    </row>
-    <row r="180" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A180" s="23">
+      <c r="A179" s="23">
         <v>42</v>
       </c>
-      <c r="B180" s="27" t="str">
+      <c r="B179" s="27" t="str">
         <f>B13</f>
         <v>Current Month Delinquency</v>
       </c>
     </row>
+    <row r="180" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A180" s="22">
+        <v>42</v>
+      </c>
+      <c r="B180" s="14" t="s">
+        <v>173</v>
+      </c>
+    </row>
     <row r="181" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A181" s="22">
-        <v>42</v>
-      </c>
-      <c r="B181" s="14" t="s">
-        <v>173</v>
+      <c r="A181" s="23">
+        <v>11</v>
+      </c>
+      <c r="B181" s="17" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="182" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A182" s="23">
-        <v>11</v>
-      </c>
-      <c r="B182" s="17" t="s">
-        <v>174</v>
+      <c r="A182" s="22">
+        <v>11</v>
+      </c>
+      <c r="B182" s="14" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="183" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A183" s="22">
-        <v>11</v>
-      </c>
-      <c r="B183" s="14" t="s">
-        <v>175</v>
+      <c r="A183" s="23">
+        <v>55</v>
+      </c>
+      <c r="B183" s="17" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="184" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A184" s="23">
-        <v>55</v>
-      </c>
-      <c r="B184" s="17" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="185" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A185" s="22">
-        <v>41</v>
-      </c>
-      <c r="B185" s="30" t="str">
+      <c r="A184" s="22">
+        <v>41</v>
+      </c>
+      <c r="B184" s="30" t="str">
         <f>B17</f>
         <v>Other Income</v>
       </c>
     </row>
-    <row r="186" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A186" s="31">
+    <row r="185" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A185" s="31">
         <v>42</v>
       </c>
-      <c r="B186" s="32" t="str">
+      <c r="B185" s="32" t="str">
         <f>B18</f>
         <v>Insufficient Notice</v>
+      </c>
+    </row>
+    <row r="186" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A186" s="1">
+        <v>110</v>
+      </c>
+      <c r="B186" s="2" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="187" spans="1:2" x14ac:dyDescent="0.25">
@@ -2810,23 +2809,23 @@
         <v>110</v>
       </c>
       <c r="B187" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="188" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A188" s="1">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="B188" s="2" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="189" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A189" s="1">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="B189" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="190" spans="1:2" x14ac:dyDescent="0.25">
@@ -2834,7 +2833,7 @@
         <v>115</v>
       </c>
       <c r="B190" s="2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="191" spans="1:2" x14ac:dyDescent="0.25">
@@ -2842,7 +2841,7 @@
         <v>115</v>
       </c>
       <c r="B191" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="192" spans="1:2" x14ac:dyDescent="0.25">
@@ -2850,23 +2849,23 @@
         <v>115</v>
       </c>
       <c r="B192" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="193" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A193" s="1">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="B193" s="2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="194" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A194" s="1">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="B194" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="195" spans="1:2" x14ac:dyDescent="0.25">
@@ -2874,47 +2873,47 @@
         <v>115</v>
       </c>
       <c r="B195" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="196" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A196" s="1">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="B196" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="197" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A197" s="1">
-        <v>121</v>
+        <v>142</v>
       </c>
       <c r="B197" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="198" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A198" s="1">
-        <v>142</v>
+        <v>160</v>
       </c>
       <c r="B198" s="2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="199" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A199" s="1">
-        <v>160</v>
+        <v>140</v>
       </c>
       <c r="B199" s="2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="200" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A200" s="1">
-        <v>140</v>
+        <v>160</v>
       </c>
       <c r="B200" s="2" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="201" spans="1:2" x14ac:dyDescent="0.25">
@@ -2922,7 +2921,7 @@
         <v>160</v>
       </c>
       <c r="B201" s="2" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="202" spans="1:2" x14ac:dyDescent="0.25">
@@ -2930,23 +2929,23 @@
         <v>160</v>
       </c>
       <c r="B202" s="2" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="203" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A203" s="1">
-        <v>160</v>
+        <v>141</v>
       </c>
       <c r="B203" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="204" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A204" s="1">
-        <v>141</v>
+        <v>160</v>
       </c>
       <c r="B204" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="205" spans="1:2" x14ac:dyDescent="0.25">
@@ -2954,7 +2953,7 @@
         <v>160</v>
       </c>
       <c r="B205" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="206" spans="1:2" x14ac:dyDescent="0.25">
@@ -2962,7 +2961,7 @@
         <v>160</v>
       </c>
       <c r="B206" s="2" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="207" spans="1:2" x14ac:dyDescent="0.25">
@@ -2970,7 +2969,7 @@
         <v>160</v>
       </c>
       <c r="B207" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="208" spans="1:2" x14ac:dyDescent="0.25">
@@ -2978,7 +2977,7 @@
         <v>160</v>
       </c>
       <c r="B208" s="2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="209" spans="1:2" x14ac:dyDescent="0.25">
@@ -2986,7 +2985,7 @@
         <v>160</v>
       </c>
       <c r="B209" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="210" spans="1:2" x14ac:dyDescent="0.25">
@@ -2994,7 +2993,7 @@
         <v>160</v>
       </c>
       <c r="B210" s="2" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="211" spans="1:2" x14ac:dyDescent="0.25">
@@ -3002,31 +3001,31 @@
         <v>160</v>
       </c>
       <c r="B211" s="2" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="212" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A212" s="1">
-        <v>160</v>
+        <v>103</v>
       </c>
       <c r="B212" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="213" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A213" s="1">
-        <v>103</v>
+        <v>160</v>
       </c>
       <c r="B213" s="2" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="214" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A214" s="1">
-        <v>160</v>
+        <v>103</v>
       </c>
       <c r="B214" s="2" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="215" spans="1:2" x14ac:dyDescent="0.25">
@@ -3034,7 +3033,7 @@
         <v>103</v>
       </c>
       <c r="B215" s="2" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="216" spans="1:2" x14ac:dyDescent="0.25">
@@ -3042,15 +3041,15 @@
         <v>103</v>
       </c>
       <c r="B216" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="217" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A217" s="1">
-        <v>103</v>
+        <v>41</v>
       </c>
       <c r="B217" s="2" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="218" spans="1:2" x14ac:dyDescent="0.25">
@@ -3058,7 +3057,7 @@
         <v>41</v>
       </c>
       <c r="B218" s="2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="219" spans="1:2" x14ac:dyDescent="0.25">
@@ -3066,7 +3065,7 @@
         <v>41</v>
       </c>
       <c r="B219" s="2" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="220" spans="1:2" x14ac:dyDescent="0.25">
@@ -3074,7 +3073,7 @@
         <v>41</v>
       </c>
       <c r="B220" s="2" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="221" spans="1:2" x14ac:dyDescent="0.25">
@@ -3082,7 +3081,7 @@
         <v>41</v>
       </c>
       <c r="B221" s="2" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="222" spans="1:2" x14ac:dyDescent="0.25">
@@ -3090,7 +3089,7 @@
         <v>41</v>
       </c>
       <c r="B222" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="223" spans="1:2" x14ac:dyDescent="0.25">
@@ -3098,7 +3097,7 @@
         <v>41</v>
       </c>
       <c r="B223" s="2" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="224" spans="1:2" x14ac:dyDescent="0.25">
@@ -3106,7 +3105,7 @@
         <v>41</v>
       </c>
       <c r="B224" s="2" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="225" spans="1:2" x14ac:dyDescent="0.25">
@@ -3114,7 +3113,7 @@
         <v>41</v>
       </c>
       <c r="B225" s="2" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="226" spans="1:2" x14ac:dyDescent="0.25">
@@ -3122,7 +3121,7 @@
         <v>41</v>
       </c>
       <c r="B226" s="2" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="227" spans="1:2" x14ac:dyDescent="0.25">
@@ -3130,15 +3129,15 @@
         <v>41</v>
       </c>
       <c r="B227" s="2" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="228" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A228" s="1">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B228" s="2" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="229" spans="1:2" x14ac:dyDescent="0.25">
@@ -3146,7 +3145,7 @@
         <v>42</v>
       </c>
       <c r="B229" s="2" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="230" spans="1:2" x14ac:dyDescent="0.25">
@@ -3154,7 +3153,7 @@
         <v>42</v>
       </c>
       <c r="B230" s="2" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="231" spans="1:2" x14ac:dyDescent="0.25">
@@ -3162,7 +3161,7 @@
         <v>42</v>
       </c>
       <c r="B231" s="2" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="232" spans="1:2" x14ac:dyDescent="0.25">
@@ -3170,7 +3169,7 @@
         <v>42</v>
       </c>
       <c r="B232" s="2" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="233" spans="1:2" x14ac:dyDescent="0.25">
@@ -3178,7 +3177,7 @@
         <v>42</v>
       </c>
       <c r="B233" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="234" spans="1:2" x14ac:dyDescent="0.25">
@@ -3186,7 +3185,7 @@
         <v>42</v>
       </c>
       <c r="B234" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="235" spans="1:2" x14ac:dyDescent="0.25">
@@ -3194,7 +3193,7 @@
         <v>42</v>
       </c>
       <c r="B235" s="2" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="236" spans="1:2" x14ac:dyDescent="0.25">
@@ -3202,7 +3201,7 @@
         <v>42</v>
       </c>
       <c r="B236" s="2" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="237" spans="1:2" x14ac:dyDescent="0.25">
@@ -3210,15 +3209,15 @@
         <v>42</v>
       </c>
       <c r="B237" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="238" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A238" s="1">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B238" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="239" spans="1:2" x14ac:dyDescent="0.25">
@@ -3226,7 +3225,7 @@
         <v>43</v>
       </c>
       <c r="B239" s="2" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="240" spans="1:2" x14ac:dyDescent="0.25">
@@ -3234,7 +3233,7 @@
         <v>43</v>
       </c>
       <c r="B240" s="2" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="241" spans="1:2" x14ac:dyDescent="0.25">
@@ -3242,7 +3241,7 @@
         <v>43</v>
       </c>
       <c r="B241" s="2" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="242" spans="1:2" x14ac:dyDescent="0.25">
@@ -3250,7 +3249,7 @@
         <v>43</v>
       </c>
       <c r="B242" s="2" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="243" spans="1:2" x14ac:dyDescent="0.25">
@@ -3258,7 +3257,7 @@
         <v>43</v>
       </c>
       <c r="B243" s="2" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="244" spans="1:2" x14ac:dyDescent="0.25">
@@ -3266,7 +3265,7 @@
         <v>43</v>
       </c>
       <c r="B244" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="245" spans="1:2" x14ac:dyDescent="0.25">
@@ -3274,7 +3273,7 @@
         <v>43</v>
       </c>
       <c r="B245" s="2" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="246" spans="1:2" x14ac:dyDescent="0.25">
@@ -3282,7 +3281,7 @@
         <v>43</v>
       </c>
       <c r="B246" s="2" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="247" spans="1:2" x14ac:dyDescent="0.25">
@@ -3290,31 +3289,31 @@
         <v>43</v>
       </c>
       <c r="B247" s="2" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="248" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A248" s="1">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="B248" s="2" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="249" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A249" s="1">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B249" s="2" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="250" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A250" s="1">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B250" s="2" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="251" spans="1:2" x14ac:dyDescent="0.25">
@@ -3322,7 +3321,7 @@
         <v>12</v>
       </c>
       <c r="B251" s="2" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="252" spans="1:2" x14ac:dyDescent="0.25">
@@ -3330,15 +3329,15 @@
         <v>12</v>
       </c>
       <c r="B252" s="2" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="253" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A253" s="1">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B253" s="2" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="254" spans="1:2" x14ac:dyDescent="0.25">
@@ -3346,39 +3345,39 @@
         <v>11</v>
       </c>
       <c r="B254" s="2" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="255" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A255" s="1">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B255" s="2" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="256" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A256" s="1">
-        <v>13</v>
+        <v>41</v>
       </c>
       <c r="B256" s="2" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="257" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A257" s="1">
-        <v>41</v>
+        <v>13</v>
       </c>
       <c r="B257" s="2" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="258" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A258" s="1">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B258" s="2" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="259" spans="1:2" x14ac:dyDescent="0.25">
@@ -3386,7 +3385,7 @@
         <v>11</v>
       </c>
       <c r="B259" s="2" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="260" spans="1:2" x14ac:dyDescent="0.25">
@@ -3394,7 +3393,7 @@
         <v>11</v>
       </c>
       <c r="B260" s="2" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="261" spans="1:2" x14ac:dyDescent="0.25">
@@ -3402,7 +3401,7 @@
         <v>11</v>
       </c>
       <c r="B261" s="2" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="262" spans="1:2" x14ac:dyDescent="0.25">
@@ -3410,7 +3409,7 @@
         <v>11</v>
       </c>
       <c r="B262" s="2" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="263" spans="1:2" x14ac:dyDescent="0.25">
@@ -3418,7 +3417,7 @@
         <v>11</v>
       </c>
       <c r="B263" s="2" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="264" spans="1:2" x14ac:dyDescent="0.25">
@@ -3426,7 +3425,7 @@
         <v>11</v>
       </c>
       <c r="B264" s="2" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="265" spans="1:2" x14ac:dyDescent="0.25">
@@ -3434,7 +3433,7 @@
         <v>11</v>
       </c>
       <c r="B265" s="2" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="266" spans="1:2" x14ac:dyDescent="0.25">
@@ -3442,7 +3441,7 @@
         <v>11</v>
       </c>
       <c r="B266" s="2" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="267" spans="1:2" x14ac:dyDescent="0.25">
@@ -3450,7 +3449,7 @@
         <v>11</v>
       </c>
       <c r="B267" s="2" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="268" spans="1:2" x14ac:dyDescent="0.25">
@@ -3458,7 +3457,7 @@
         <v>11</v>
       </c>
       <c r="B268" s="2" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="269" spans="1:2" x14ac:dyDescent="0.25">
@@ -3466,7 +3465,7 @@
         <v>11</v>
       </c>
       <c r="B269" s="2" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="270" spans="1:2" x14ac:dyDescent="0.25">
@@ -3474,23 +3473,23 @@
         <v>11</v>
       </c>
       <c r="B270" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="271" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A271" s="1">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B271" s="2" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="272" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A272" s="1">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B272" s="2" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="273" spans="1:2" x14ac:dyDescent="0.25">
@@ -3498,7 +3497,7 @@
         <v>11</v>
       </c>
       <c r="B273" s="2" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="274" spans="1:2" x14ac:dyDescent="0.25">
@@ -3506,7 +3505,7 @@
         <v>11</v>
       </c>
       <c r="B274" s="2" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="275" spans="1:2" x14ac:dyDescent="0.25">
@@ -3514,7 +3513,7 @@
         <v>11</v>
       </c>
       <c r="B275" s="2" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="276" spans="1:2" x14ac:dyDescent="0.25">
@@ -3522,7 +3521,7 @@
         <v>11</v>
       </c>
       <c r="B276" s="2" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="277" spans="1:2" x14ac:dyDescent="0.25">
@@ -3530,71 +3529,71 @@
         <v>11</v>
       </c>
       <c r="B277" s="2" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
     <row r="278" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A278" s="1">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="B278" s="2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="279" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A279" s="1">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B279" s="2" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="280" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A280" s="1">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B280" s="2" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="281" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A281" s="1">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="B281" s="2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="282" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A282" s="1">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="B282" s="2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="283" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A283" s="1">
-        <v>22</v>
+        <v>41</v>
       </c>
       <c r="B283" s="2" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="284" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A284" s="1">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="B284" s="2" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="285" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A285" s="1">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B285" s="2" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="286" spans="1:2" x14ac:dyDescent="0.25">
@@ -3602,15 +3601,15 @@
         <v>22</v>
       </c>
       <c r="B286" s="2" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
     </row>
     <row r="287" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A287" s="1">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="B287" s="2" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="288" spans="1:2" x14ac:dyDescent="0.25">
@@ -3618,30 +3617,22 @@
         <v>60</v>
       </c>
       <c r="B288" s="2" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="289" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A289" s="1">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="B289" s="2" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
     <row r="290" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A290" s="1">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="B290" s="2" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="291" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A291" s="1">
-        <v>30</v>
-      </c>
-      <c r="B291" s="2" t="s">
         <v>280</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove duplicate I&E internal mappings
</commit_message>
<xml_diff>
--- a/src/lib/automation/ie/reference/To add I&E.xlsx
+++ b/src/lib/automation/ie/reference/To add I&E.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8fcd883c776305f1/Documentos/Keystone/keystone-os/src/lib/automation/ie/reference/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="11_20C4315295263003D1BD0F964BC8F3756E9CBE04" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E4ACADDF-F71B-48EE-BD48-8714C68D5F2A}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="11_20C4315295263003D1BD0F964BC8F3756E9CBE04" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{043E67DD-55A6-48FC-B722-E28DA5DCE0F5}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$2:$B$168</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -33,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="278">
   <si>
     <t>Number</t>
   </si>
@@ -71,9 +74,6 @@
     <t>Employee Discounts</t>
   </si>
   <si>
-    <t>Current Month Delinquency</t>
-  </si>
-  <si>
     <t>Prepaid Rent</t>
   </si>
   <si>
@@ -101,9 +101,6 @@
     <t>Collection Agency/Attorney</t>
   </si>
   <si>
-    <t>Cable Provider Payments</t>
-  </si>
-  <si>
     <t>Deposit Forfeitures</t>
   </si>
   <si>
@@ -528,9 +525,6 @@
   </si>
   <si>
     <t>Total Training &amp; Continuing Ed</t>
-  </si>
-  <si>
-    <t>Personal Property Taxes</t>
   </si>
   <si>
     <t>Bad Debt Expense</t>
@@ -1382,7 +1376,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:B290"/>
+  <dimension ref="A2:B284"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.28515625" customWidth="1"/>
@@ -1472,73 +1466,73 @@
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="5">
+      <c r="A13" s="15">
         <v>110</v>
       </c>
-      <c r="B13" s="14" t="s">
+      <c r="B13" s="16" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="15">
-        <v>110</v>
-      </c>
-      <c r="B14" s="16" t="s">
+      <c r="A14" s="5"/>
+      <c r="B14" s="14" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="5"/>
-      <c r="B15" s="14" t="s">
+      <c r="A15" s="15"/>
+      <c r="B15" s="17" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="15"/>
-      <c r="B16" s="17" t="s">
+      <c r="A16" s="18"/>
+      <c r="B16" s="14" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="18"/>
-      <c r="B17" s="14" t="s">
+      <c r="A17" s="15">
+        <v>160</v>
+      </c>
+      <c r="B17" s="17" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="15">
+      <c r="A18" s="12">
         <v>160</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="14" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="12">
+      <c r="A19" s="19">
         <v>160</v>
       </c>
-      <c r="B19" s="14" t="s">
+      <c r="B19" s="17" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="19">
+      <c r="A20" s="20">
         <v>160</v>
       </c>
-      <c r="B20" s="17" t="s">
+      <c r="B20" s="14" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="20">
+      <c r="A21" s="21">
         <v>160</v>
       </c>
-      <c r="B21" s="14" t="s">
+      <c r="B21" s="17" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="21">
+      <c r="A22" s="23">
         <v>160</v>
       </c>
       <c r="B22" s="17" t="s">
@@ -1595,7 +1589,7 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="22">
-        <v>160</v>
+        <v>140</v>
       </c>
       <c r="B29" s="14" t="s">
         <v>28</v>
@@ -1611,7 +1605,7 @@
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="22">
-        <v>140</v>
+        <v>160</v>
       </c>
       <c r="B31" s="14" t="s">
         <v>30</v>
@@ -1627,7 +1621,7 @@
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="22">
-        <v>160</v>
+        <v>103</v>
       </c>
       <c r="B33" s="14" t="s">
         <v>32</v>
@@ -1635,25 +1629,21 @@
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="23">
-        <v>160</v>
+        <v>103</v>
       </c>
       <c r="B34" s="17" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A35" s="22">
-        <v>103</v>
-      </c>
+      <c r="A35" s="22"/>
       <c r="B35" s="14" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A36" s="23">
-        <v>103</v>
-      </c>
-      <c r="B36" s="17" t="s">
+      <c r="A36" s="24"/>
+      <c r="B36" s="16" t="s">
         <v>35</v>
       </c>
     </row>
@@ -1664,19 +1654,23 @@
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38" s="24"/>
+      <c r="A38" s="23"/>
       <c r="B38" s="16" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A39" s="22"/>
+      <c r="A39" s="22">
+        <v>41</v>
+      </c>
       <c r="B39" s="14" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A40" s="23"/>
+      <c r="A40" s="23">
+        <v>41</v>
+      </c>
       <c r="B40" s="16" t="s">
         <v>39</v>
       </c>
@@ -1693,12 +1687,12 @@
       <c r="A42" s="23">
         <v>41</v>
       </c>
-      <c r="B42" s="16" t="s">
+      <c r="B42" s="17" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A43" s="22">
+      <c r="A43" s="25">
         <v>41</v>
       </c>
       <c r="B43" s="14" t="s">
@@ -1706,7 +1700,7 @@
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A44" s="23">
+      <c r="A44" s="24">
         <v>41</v>
       </c>
       <c r="B44" s="17" t="s">
@@ -1722,7 +1716,7 @@
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A46" s="24">
+      <c r="A46" s="23">
         <v>41</v>
       </c>
       <c r="B46" s="17" t="s">
@@ -1730,7 +1724,7 @@
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A47" s="25">
+      <c r="A47" s="22">
         <v>41</v>
       </c>
       <c r="B47" s="14" t="s">
@@ -1738,7 +1732,7 @@
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A48" s="23">
+      <c r="A48" s="24">
         <v>41</v>
       </c>
       <c r="B48" s="17" t="s">
@@ -1754,7 +1748,7 @@
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A50" s="24">
+      <c r="A50" s="23">
         <v>41</v>
       </c>
       <c r="B50" s="17" t="s">
@@ -1842,30 +1836,30 @@
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A61" s="22">
-        <v>41</v>
-      </c>
+      <c r="A61" s="22"/>
       <c r="B61" s="14" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A62" s="23">
-        <v>41</v>
-      </c>
+      <c r="A62" s="23"/>
       <c r="B62" s="17" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A63" s="22"/>
+      <c r="A63" s="22">
+        <v>43</v>
+      </c>
       <c r="B63" s="14" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A64" s="23"/>
-      <c r="B64" s="17" t="s">
+      <c r="A64" s="23">
+        <v>43</v>
+      </c>
+      <c r="B64" s="16" t="s">
         <v>63</v>
       </c>
     </row>
@@ -1926,29 +1920,29 @@
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A72" s="23">
-        <v>43</v>
-      </c>
+      <c r="A72" s="23"/>
       <c r="B72" s="16" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A73" s="22">
-        <v>43</v>
-      </c>
+      <c r="A73" s="22"/>
       <c r="B73" s="14" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A74" s="23"/>
-      <c r="B74" s="16" t="s">
+      <c r="A74" s="23">
+        <v>11</v>
+      </c>
+      <c r="B74" s="17" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A75" s="22"/>
+      <c r="A75" s="22">
+        <v>11</v>
+      </c>
       <c r="B75" s="14" t="s">
         <v>74</v>
       </c>
@@ -1963,7 +1957,7 @@
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77" s="22">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B77" s="14" t="s">
         <v>76</v>
@@ -1971,7 +1965,7 @@
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78" s="23">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B78" s="17" t="s">
         <v>77</v>
@@ -1979,7 +1973,7 @@
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79" s="22">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B79" s="14" t="s">
         <v>78</v>
@@ -1987,7 +1981,7 @@
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80" s="23">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B80" s="17" t="s">
         <v>79</v>
@@ -2042,29 +2036,29 @@
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A87" s="22">
-        <v>11</v>
-      </c>
+      <c r="A87" s="22"/>
       <c r="B87" s="14" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A88" s="23">
-        <v>11</v>
-      </c>
+      <c r="A88" s="23"/>
       <c r="B88" s="17" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A89" s="22"/>
+      <c r="A89" s="22">
+        <v>12</v>
+      </c>
       <c r="B89" s="14" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A90" s="23"/>
+      <c r="A90" s="23">
+        <v>12</v>
+      </c>
       <c r="B90" s="17" t="s">
         <v>89</v>
       </c>
@@ -2073,23 +2067,23 @@
       <c r="A91" s="22">
         <v>12</v>
       </c>
-      <c r="B91" s="14" t="s">
+      <c r="B91" s="26" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92" s="23">
-        <v>12</v>
-      </c>
-      <c r="B92" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="B92" s="16" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93" s="22">
-        <v>12</v>
-      </c>
-      <c r="B93" s="26" t="s">
+        <v>15</v>
+      </c>
+      <c r="B93" s="14" t="s">
         <v>92</v>
       </c>
     </row>
@@ -2103,7 +2097,7 @@
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A95" s="22">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B95" s="14" t="s">
         <v>94</v>
@@ -2111,7 +2105,7 @@
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A96" s="23">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B96" s="16" t="s">
         <v>95</v>
@@ -2119,7 +2113,7 @@
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97" s="22">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B97" s="14" t="s">
         <v>96</v>
@@ -2127,7 +2121,7 @@
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A98" s="23">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B98" s="16" t="s">
         <v>97</v>
@@ -2135,17 +2129,17 @@
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A99" s="22">
-        <v>13</v>
-      </c>
-      <c r="B99" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="B99" s="26" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A100" s="23">
-        <v>12</v>
-      </c>
-      <c r="B100" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="B100" s="17" t="s">
         <v>99</v>
       </c>
     </row>
@@ -2158,8 +2152,8 @@
       </c>
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A102" s="23">
-        <v>11</v>
+      <c r="A102" s="24">
+        <v>13</v>
       </c>
       <c r="B102" s="17" t="s">
         <v>101</v>
@@ -2167,24 +2161,20 @@
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A103" s="22">
-        <v>11</v>
-      </c>
-      <c r="B103" s="26" t="s">
+        <v>16</v>
+      </c>
+      <c r="B103" s="14" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A104" s="24">
-        <v>13</v>
-      </c>
+      <c r="A104" s="23"/>
       <c r="B104" s="17" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A105" s="22">
-        <v>16</v>
-      </c>
+      <c r="A105" s="22"/>
       <c r="B105" s="14" t="s">
         <v>104</v>
       </c>
@@ -2196,13 +2186,17 @@
       </c>
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A107" s="22"/>
+      <c r="A107" s="22">
+        <v>42</v>
+      </c>
       <c r="B107" s="14" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A108" s="23"/>
+      <c r="A108" s="23">
+        <v>42</v>
+      </c>
       <c r="B108" s="17" t="s">
         <v>107</v>
       </c>
@@ -2211,7 +2205,7 @@
       <c r="A109" s="22">
         <v>42</v>
       </c>
-      <c r="B109" s="14" t="s">
+      <c r="B109" s="26" t="s">
         <v>108</v>
       </c>
     </row>
@@ -2275,7 +2269,7 @@
       <c r="A117" s="22">
         <v>42</v>
       </c>
-      <c r="B117" s="26" t="s">
+      <c r="B117" s="14" t="s">
         <v>116</v>
       </c>
     </row>
@@ -2283,7 +2277,7 @@
       <c r="A118" s="23">
         <v>42</v>
       </c>
-      <c r="B118" s="17" t="s">
+      <c r="B118" s="27" t="s">
         <v>117</v>
       </c>
     </row>
@@ -2299,7 +2293,7 @@
       <c r="A120" s="23">
         <v>42</v>
       </c>
-      <c r="B120" s="27" t="s">
+      <c r="B120" s="17" t="s">
         <v>119</v>
       </c>
     </row>
@@ -2312,30 +2306,30 @@
       </c>
     </row>
     <row r="122" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A122" s="23">
-        <v>42</v>
-      </c>
+      <c r="A122" s="23"/>
       <c r="B122" s="17" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="123" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A123" s="22">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="B123" s="14" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="124" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A124" s="23"/>
+      <c r="A124" s="23">
+        <v>21</v>
+      </c>
       <c r="B124" s="17" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="125" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A125" s="22">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B125" s="14" t="s">
         <v>124</v>
@@ -2343,7 +2337,7 @@
     </row>
     <row r="126" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A126" s="23">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B126" s="17" t="s">
         <v>125</v>
@@ -2351,7 +2345,7 @@
     </row>
     <row r="127" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A127" s="22">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B127" s="14" t="s">
         <v>126</v>
@@ -2359,69 +2353,69 @@
     </row>
     <row r="128" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A128" s="23">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B128" s="17" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="129" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A129" s="22">
-        <v>22</v>
-      </c>
+      <c r="A129" s="25"/>
       <c r="B129" s="14" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="130" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A130" s="23">
-        <v>22</v>
-      </c>
+      <c r="A130" s="23"/>
       <c r="B130" s="17" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="131" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A131" s="25"/>
+      <c r="A131" s="22">
+        <v>30</v>
+      </c>
       <c r="B131" s="14" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="132" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A132" s="23"/>
       <c r="B132" s="17" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="133" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A133" s="22">
-        <v>30</v>
-      </c>
+      <c r="A133" s="20"/>
       <c r="B133" s="14" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="134" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A134" s="23"/>
+      <c r="A134" s="21"/>
       <c r="B134" s="17" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="135" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A135" s="20"/>
+      <c r="A135" s="22">
+        <v>50</v>
+      </c>
       <c r="B135" s="14" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="136" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A136" s="21"/>
+      <c r="A136" s="23">
+        <v>41</v>
+      </c>
       <c r="B136" s="17" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="137" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A137" s="22">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="B137" s="14" t="s">
         <v>135</v>
@@ -2429,7 +2423,7 @@
     </row>
     <row r="138" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A138" s="23">
-        <v>41</v>
+        <v>60</v>
       </c>
       <c r="B138" s="17" t="s">
         <v>136</v>
@@ -2444,380 +2438,380 @@
       </c>
     </row>
     <row r="140" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A140" s="23">
-        <v>60</v>
-      </c>
+      <c r="A140" s="23"/>
       <c r="B140" s="17" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="141" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A141" s="22">
-        <v>41</v>
-      </c>
+      <c r="A141" s="22"/>
       <c r="B141" s="14" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="142" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A142" s="23"/>
+      <c r="A142" s="24">
+        <v>111</v>
+      </c>
       <c r="B142" s="17" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="143" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A143" s="22"/>
+      <c r="A143" s="22">
+        <v>41</v>
+      </c>
       <c r="B143" s="14" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="144" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A144" s="24">
-        <v>111</v>
+      <c r="A144" s="23">
+        <v>55</v>
       </c>
       <c r="B144" s="17" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="145" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A145" s="22">
-        <v>41</v>
-      </c>
-      <c r="B145" s="14" t="s">
+      <c r="A145" s="28">
+        <v>115</v>
+      </c>
+      <c r="B145" s="6" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="146" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A146" s="23">
-        <v>55</v>
-      </c>
-      <c r="B146" s="17" t="s">
+      <c r="A146" s="22">
+        <v>142</v>
+      </c>
+      <c r="B146" s="14" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="147" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A147" s="28">
-        <v>115</v>
-      </c>
-      <c r="B147" s="6" t="s">
+      <c r="A147" s="23">
+        <v>160</v>
+      </c>
+      <c r="B147" s="17" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="148" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A148" s="23">
-        <v>142</v>
-      </c>
-      <c r="B148" s="17" t="s">
+      <c r="A148" s="22">
+        <v>41</v>
+      </c>
+      <c r="B148" s="26" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A149" s="23">
+        <v>41</v>
+      </c>
+      <c r="B149" s="16" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A150" s="22">
+        <v>24</v>
+      </c>
+      <c r="B150" s="14" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A151" s="23">
+        <v>11</v>
+      </c>
+      <c r="B151" s="17" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A152" s="22">
+        <v>11</v>
+      </c>
+      <c r="B152" s="14" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A153" s="23">
+        <v>11</v>
+      </c>
+      <c r="B153" s="17" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A154" s="22">
+        <v>11</v>
+      </c>
+      <c r="B154" s="14" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A155" s="23">
+        <v>11</v>
+      </c>
+      <c r="B155" s="17" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="156" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A156" s="22">
+        <v>11</v>
+      </c>
+      <c r="B156" s="14" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A157" s="23">
+        <v>11</v>
+      </c>
+      <c r="B157" s="17" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A158" s="22">
+        <v>12</v>
+      </c>
+      <c r="B158" s="14" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="159" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A159" s="23">
+        <v>16</v>
+      </c>
+      <c r="B159" s="16" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A160" s="22">
+        <v>11</v>
+      </c>
+      <c r="B160" s="14" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A161" s="23"/>
+      <c r="B161" s="16" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A162" s="22"/>
+      <c r="B162" s="26" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A163" s="23"/>
+      <c r="B163" s="17" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A164" s="22"/>
+      <c r="B164" s="14" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A165" s="23">
+        <v>41</v>
+      </c>
+      <c r="B165" s="17" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A166" s="29">
+        <v>121</v>
+      </c>
+      <c r="B166" s="17" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="167" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A167" s="23">
+        <v>141</v>
+      </c>
+      <c r="B167" s="17" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="168" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A168" s="22"/>
+      <c r="B168" s="14" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A169" s="23"/>
+      <c r="B169" s="16"/>
+    </row>
+    <row r="170" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A170" s="22">
+        <v>41</v>
+      </c>
+      <c r="B170" s="26" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A171" s="23">
+        <v>41</v>
+      </c>
+      <c r="B171" s="16" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="172" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A172" s="22">
         <v>22</v>
       </c>
-    </row>
-    <row r="149" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A149" s="22">
-        <v>142</v>
-      </c>
-      <c r="B149" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="150" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A150" s="23">
-        <v>160</v>
-      </c>
-      <c r="B150" s="17" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="151" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A151" s="22">
-        <v>41</v>
-      </c>
-      <c r="B151" s="26" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="152" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A152" s="23">
-        <v>41</v>
-      </c>
-      <c r="B152" s="16" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="153" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A153" s="22">
-        <v>24</v>
-      </c>
-      <c r="B153" s="14" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="154" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A154" s="23">
-        <v>11</v>
-      </c>
-      <c r="B154" s="17" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="155" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A155" s="22">
-        <v>11</v>
-      </c>
-      <c r="B155" s="14" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="156" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A156" s="23">
-        <v>11</v>
-      </c>
-      <c r="B156" s="17" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="157" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A157" s="22">
-        <v>11</v>
-      </c>
-      <c r="B157" s="14" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="158" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A158" s="23">
-        <v>11</v>
-      </c>
-      <c r="B158" s="17" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="159" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A159" s="22">
-        <v>11</v>
-      </c>
-      <c r="B159" s="14" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="160" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A160" s="23">
-        <v>11</v>
-      </c>
-      <c r="B160" s="17" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="161" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A161" s="22">
-        <v>12</v>
-      </c>
-      <c r="B161" s="14" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="162" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A162" s="23">
-        <v>16</v>
-      </c>
-      <c r="B162" s="16" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="163" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A163" s="22">
-        <v>11</v>
-      </c>
-      <c r="B163" s="14" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="164" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A164" s="23"/>
-      <c r="B164" s="16" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="165" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A165" s="22"/>
-      <c r="B165" s="26" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="166" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A166" s="23"/>
-      <c r="B166" s="17" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="167" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A167" s="22"/>
-      <c r="B167" s="14" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="168" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A168" s="23">
-        <v>41</v>
-      </c>
-      <c r="B168" s="17" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="169" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A169" s="22">
-        <v>41</v>
-      </c>
-      <c r="B169" s="14" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="170" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A170" s="29">
-        <v>121</v>
-      </c>
-      <c r="B170" s="17" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="171" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A171" s="28">
-        <v>121</v>
-      </c>
-      <c r="B171" s="14" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="172" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A172" s="23">
-        <v>141</v>
-      </c>
-      <c r="B172" s="17" t="s">
-        <v>167</v>
+      <c r="B172" s="14" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="173" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A173" s="22"/>
-      <c r="B173" s="14" t="s">
-        <v>168</v>
+      <c r="A173" s="23">
+        <v>30</v>
+      </c>
+      <c r="B173" s="17" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="174" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A174" s="23"/>
-      <c r="B174" s="16"/>
+      <c r="A174" s="23">
+        <v>42</v>
+      </c>
+      <c r="B174" s="27" t="e">
+        <f>#REF!</f>
+        <v>#REF!</v>
+      </c>
     </row>
     <row r="175" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A175" s="22">
-        <v>41</v>
-      </c>
-      <c r="B175" s="26" t="s">
-        <v>169</v>
+        <v>42</v>
+      </c>
+      <c r="B175" s="14" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="176" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A176" s="23">
-        <v>41</v>
-      </c>
-      <c r="B176" s="16" t="s">
-        <v>170</v>
+        <v>11</v>
+      </c>
+      <c r="B176" s="17" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="177" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A177" s="22">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="B177" s="14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="178" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A178" s="23">
-        <v>30</v>
-      </c>
-      <c r="B178" s="17" t="s">
-        <v>172</v>
+      <c r="A178" s="22">
+        <v>41</v>
+      </c>
+      <c r="B178" s="30" t="str">
+        <f>B16</f>
+        <v>Other Income</v>
       </c>
     </row>
     <row r="179" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A179" s="23">
+      <c r="A179" s="31">
         <v>42</v>
       </c>
-      <c r="B179" s="27" t="str">
-        <f>B13</f>
-        <v>Current Month Delinquency</v>
+      <c r="B179" s="32" t="str">
+        <f>B17</f>
+        <v>Insufficient Notice</v>
       </c>
     </row>
     <row r="180" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A180" s="22">
-        <v>42</v>
-      </c>
-      <c r="B180" s="14" t="s">
+      <c r="A180" s="1">
+        <v>110</v>
+      </c>
+      <c r="B180" s="2" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="181" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A181" s="23">
-        <v>11</v>
-      </c>
-      <c r="B181" s="17" t="s">
+      <c r="A181" s="1">
+        <v>110</v>
+      </c>
+      <c r="B181" s="2" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="182" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A182" s="22">
-        <v>11</v>
-      </c>
-      <c r="B182" s="14" t="s">
+      <c r="A182" s="1">
+        <v>120</v>
+      </c>
+      <c r="B182" s="2" t="s">
         <v>175</v>
       </c>
     </row>
     <row r="183" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A183" s="23">
-        <v>55</v>
-      </c>
-      <c r="B183" s="17" t="s">
-        <v>165</v>
+      <c r="A183" s="1">
+        <v>115</v>
+      </c>
+      <c r="B183" s="2" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="184" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A184" s="22">
-        <v>41</v>
-      </c>
-      <c r="B184" s="30" t="str">
-        <f>B17</f>
-        <v>Other Income</v>
+      <c r="A184" s="1">
+        <v>115</v>
+      </c>
+      <c r="B184" s="2" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="185" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A185" s="31">
-        <v>42</v>
-      </c>
-      <c r="B185" s="32" t="str">
-        <f>B18</f>
-        <v>Insufficient Notice</v>
+      <c r="A185" s="1">
+        <v>115</v>
+      </c>
+      <c r="B185" s="2" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="186" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A186" s="1">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="B186" s="2" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
     </row>
     <row r="187" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A187" s="1">
-        <v>110</v>
+        <v>121</v>
       </c>
       <c r="B187" s="2" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
     </row>
     <row r="188" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A188" s="1">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="B188" s="2" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
     </row>
     <row r="189" spans="1:2" x14ac:dyDescent="0.25">
@@ -2825,71 +2819,71 @@
         <v>115</v>
       </c>
       <c r="B189" s="2" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
     </row>
     <row r="190" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A190" s="1">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="B190" s="2" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
     </row>
     <row r="191" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A191" s="1">
-        <v>115</v>
+        <v>142</v>
       </c>
       <c r="B191" s="2" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
     </row>
     <row r="192" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A192" s="1">
-        <v>115</v>
+        <v>160</v>
       </c>
       <c r="B192" s="2" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="193" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A193" s="1">
-        <v>121</v>
+        <v>140</v>
       </c>
       <c r="B193" s="2" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
     </row>
     <row r="194" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A194" s="1">
-        <v>115</v>
+        <v>160</v>
       </c>
       <c r="B194" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="195" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A195" s="1">
-        <v>115</v>
+        <v>160</v>
       </c>
       <c r="B195" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
     </row>
     <row r="196" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A196" s="1">
-        <v>121</v>
+        <v>160</v>
       </c>
       <c r="B196" s="2" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
     </row>
     <row r="197" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A197" s="1">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B197" s="2" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
     </row>
     <row r="198" spans="1:2" x14ac:dyDescent="0.25">
@@ -2897,15 +2891,15 @@
         <v>160</v>
       </c>
       <c r="B198" s="2" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
     </row>
     <row r="199" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A199" s="1">
-        <v>140</v>
+        <v>160</v>
       </c>
       <c r="B199" s="2" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
     </row>
     <row r="200" spans="1:2" x14ac:dyDescent="0.25">
@@ -2913,7 +2907,7 @@
         <v>160</v>
       </c>
       <c r="B200" s="2" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
     </row>
     <row r="201" spans="1:2" x14ac:dyDescent="0.25">
@@ -2921,7 +2915,7 @@
         <v>160</v>
       </c>
       <c r="B201" s="2" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
     </row>
     <row r="202" spans="1:2" x14ac:dyDescent="0.25">
@@ -2929,15 +2923,15 @@
         <v>160</v>
       </c>
       <c r="B202" s="2" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
     </row>
     <row r="203" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A203" s="1">
-        <v>141</v>
+        <v>160</v>
       </c>
       <c r="B203" s="2" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
     </row>
     <row r="204" spans="1:2" x14ac:dyDescent="0.25">
@@ -2945,7 +2939,7 @@
         <v>160</v>
       </c>
       <c r="B204" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
     </row>
     <row r="205" spans="1:2" x14ac:dyDescent="0.25">
@@ -2953,15 +2947,15 @@
         <v>160</v>
       </c>
       <c r="B205" s="2" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
     </row>
     <row r="206" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A206" s="1">
-        <v>160</v>
+        <v>103</v>
       </c>
       <c r="B206" s="2" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
     </row>
     <row r="207" spans="1:2" x14ac:dyDescent="0.25">
@@ -2969,79 +2963,79 @@
         <v>160</v>
       </c>
       <c r="B207" s="2" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
     </row>
     <row r="208" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A208" s="1">
-        <v>160</v>
+        <v>103</v>
       </c>
       <c r="B208" s="2" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
     </row>
     <row r="209" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A209" s="1">
-        <v>160</v>
+        <v>103</v>
       </c>
       <c r="B209" s="2" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
     </row>
     <row r="210" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A210" s="1">
-        <v>160</v>
+        <v>103</v>
       </c>
       <c r="B210" s="2" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
     </row>
     <row r="211" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A211" s="1">
-        <v>160</v>
+        <v>41</v>
       </c>
       <c r="B211" s="2" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
     </row>
     <row r="212" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A212" s="1">
-        <v>103</v>
+        <v>41</v>
       </c>
       <c r="B212" s="2" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
     </row>
     <row r="213" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A213" s="1">
-        <v>160</v>
+        <v>41</v>
       </c>
       <c r="B213" s="2" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
     </row>
     <row r="214" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A214" s="1">
-        <v>103</v>
+        <v>41</v>
       </c>
       <c r="B214" s="2" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
     </row>
     <row r="215" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A215" s="1">
-        <v>103</v>
+        <v>41</v>
       </c>
       <c r="B215" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="216" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A216" s="1">
-        <v>103</v>
+        <v>41</v>
       </c>
       <c r="B216" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
     </row>
     <row r="217" spans="1:2" x14ac:dyDescent="0.25">
@@ -3049,7 +3043,7 @@
         <v>41</v>
       </c>
       <c r="B217" s="2" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
     </row>
     <row r="218" spans="1:2" x14ac:dyDescent="0.25">
@@ -3057,7 +3051,7 @@
         <v>41</v>
       </c>
       <c r="B218" s="2" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
     </row>
     <row r="219" spans="1:2" x14ac:dyDescent="0.25">
@@ -3065,7 +3059,7 @@
         <v>41</v>
       </c>
       <c r="B219" s="2" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
     </row>
     <row r="220" spans="1:2" x14ac:dyDescent="0.25">
@@ -3073,7 +3067,7 @@
         <v>41</v>
       </c>
       <c r="B220" s="2" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
     </row>
     <row r="221" spans="1:2" x14ac:dyDescent="0.25">
@@ -3081,55 +3075,55 @@
         <v>41</v>
       </c>
       <c r="B221" s="2" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
     </row>
     <row r="222" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A222" s="1">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B222" s="2" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
     </row>
     <row r="223" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A223" s="1">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B223" s="2" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
     </row>
     <row r="224" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A224" s="1">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B224" s="2" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="225" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A225" s="1">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B225" s="2" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="226" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A226" s="1">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B226" s="2" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
     </row>
     <row r="227" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A227" s="1">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B227" s="2" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
     </row>
     <row r="228" spans="1:2" x14ac:dyDescent="0.25">
@@ -3137,7 +3131,7 @@
         <v>42</v>
       </c>
       <c r="B228" s="2" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
     </row>
     <row r="229" spans="1:2" x14ac:dyDescent="0.25">
@@ -3145,7 +3139,7 @@
         <v>42</v>
       </c>
       <c r="B229" s="2" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
     </row>
     <row r="230" spans="1:2" x14ac:dyDescent="0.25">
@@ -3153,7 +3147,7 @@
         <v>42</v>
       </c>
       <c r="B230" s="2" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
     </row>
     <row r="231" spans="1:2" x14ac:dyDescent="0.25">
@@ -3161,55 +3155,55 @@
         <v>42</v>
       </c>
       <c r="B231" s="2" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
     </row>
     <row r="232" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A232" s="1">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B232" s="2" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
     </row>
     <row r="233" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A233" s="1">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B233" s="2" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
     </row>
     <row r="234" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A234" s="1">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B234" s="2" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
     </row>
     <row r="235" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A235" s="1">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B235" s="2" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
     </row>
     <row r="236" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A236" s="1">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B236" s="2" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
     </row>
     <row r="237" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A237" s="1">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B237" s="2" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
     </row>
     <row r="238" spans="1:2" x14ac:dyDescent="0.25">
@@ -3217,7 +3211,7 @@
         <v>43</v>
       </c>
       <c r="B238" s="2" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
     </row>
     <row r="239" spans="1:2" x14ac:dyDescent="0.25">
@@ -3225,7 +3219,7 @@
         <v>43</v>
       </c>
       <c r="B239" s="2" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
     </row>
     <row r="240" spans="1:2" x14ac:dyDescent="0.25">
@@ -3233,7 +3227,7 @@
         <v>43</v>
       </c>
       <c r="B240" s="2" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
     </row>
     <row r="241" spans="1:2" x14ac:dyDescent="0.25">
@@ -3241,95 +3235,95 @@
         <v>43</v>
       </c>
       <c r="B241" s="2" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
     </row>
     <row r="242" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A242" s="1">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="B242" s="2" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
     </row>
     <row r="243" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A243" s="1">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="B243" s="2" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
     </row>
     <row r="244" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A244" s="1">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="B244" s="2" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
     </row>
     <row r="245" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A245" s="1">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="B245" s="2" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
     </row>
     <row r="246" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A246" s="1">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="B246" s="2" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
     </row>
     <row r="247" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A247" s="1">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="B247" s="2" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
     </row>
     <row r="248" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A248" s="1">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B248" s="2" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
     </row>
     <row r="249" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A249" s="1">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B249" s="2" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
     </row>
     <row r="250" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A250" s="1">
-        <v>12</v>
+        <v>41</v>
       </c>
       <c r="B250" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
     </row>
     <row r="251" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A251" s="1">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B251" s="2" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
     </row>
     <row r="252" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A252" s="1">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B252" s="2" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="253" spans="1:2" x14ac:dyDescent="0.25">
@@ -3337,7 +3331,7 @@
         <v>11</v>
       </c>
       <c r="B253" s="2" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
     </row>
     <row r="254" spans="1:2" x14ac:dyDescent="0.25">
@@ -3345,31 +3339,31 @@
         <v>11</v>
       </c>
       <c r="B254" s="2" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
     </row>
     <row r="255" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A255" s="1">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B255" s="2" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="256" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A256" s="1">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="B256" s="2" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
     </row>
     <row r="257" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A257" s="1">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B257" s="2" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
     </row>
     <row r="258" spans="1:2" x14ac:dyDescent="0.25">
@@ -3377,7 +3371,7 @@
         <v>11</v>
       </c>
       <c r="B258" s="2" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
     </row>
     <row r="259" spans="1:2" x14ac:dyDescent="0.25">
@@ -3385,7 +3379,7 @@
         <v>11</v>
       </c>
       <c r="B259" s="2" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
     </row>
     <row r="260" spans="1:2" x14ac:dyDescent="0.25">
@@ -3393,7 +3387,7 @@
         <v>11</v>
       </c>
       <c r="B260" s="2" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="261" spans="1:2" x14ac:dyDescent="0.25">
@@ -3401,7 +3395,7 @@
         <v>11</v>
       </c>
       <c r="B261" s="2" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="262" spans="1:2" x14ac:dyDescent="0.25">
@@ -3409,7 +3403,7 @@
         <v>11</v>
       </c>
       <c r="B262" s="2" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="263" spans="1:2" x14ac:dyDescent="0.25">
@@ -3417,7 +3411,7 @@
         <v>11</v>
       </c>
       <c r="B263" s="2" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
     </row>
     <row r="264" spans="1:2" x14ac:dyDescent="0.25">
@@ -3425,15 +3419,15 @@
         <v>11</v>
       </c>
       <c r="B264" s="2" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
     </row>
     <row r="265" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A265" s="1">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B265" s="2" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
     </row>
     <row r="266" spans="1:2" x14ac:dyDescent="0.25">
@@ -3441,7 +3435,7 @@
         <v>11</v>
       </c>
       <c r="B266" s="2" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
     </row>
     <row r="267" spans="1:2" x14ac:dyDescent="0.25">
@@ -3449,7 +3443,7 @@
         <v>11</v>
       </c>
       <c r="B267" s="2" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
     </row>
     <row r="268" spans="1:2" x14ac:dyDescent="0.25">
@@ -3457,7 +3451,7 @@
         <v>11</v>
       </c>
       <c r="B268" s="2" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
     </row>
     <row r="269" spans="1:2" x14ac:dyDescent="0.25">
@@ -3465,7 +3459,7 @@
         <v>11</v>
       </c>
       <c r="B269" s="2" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
     </row>
     <row r="270" spans="1:2" x14ac:dyDescent="0.25">
@@ -3473,79 +3467,79 @@
         <v>11</v>
       </c>
       <c r="B270" s="2" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
     </row>
     <row r="271" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A271" s="1">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B271" s="2" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
     </row>
     <row r="272" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A272" s="1">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="B272" s="2" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
     </row>
     <row r="273" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A273" s="1">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="B273" s="2" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
     </row>
     <row r="274" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A274" s="1">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="B274" s="2" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
     </row>
     <row r="275" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A275" s="1">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="B275" s="2" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
     </row>
     <row r="276" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A276" s="1">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="B276" s="2" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
     </row>
     <row r="277" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A277" s="1">
-        <v>11</v>
+        <v>41</v>
       </c>
       <c r="B277" s="2" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
     </row>
     <row r="278" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A278" s="1">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B278" s="2" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
     </row>
     <row r="279" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A279" s="1">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B279" s="2" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
     </row>
     <row r="280" spans="1:2" x14ac:dyDescent="0.25">
@@ -3553,87 +3547,39 @@
         <v>22</v>
       </c>
       <c r="B280" s="2" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
     </row>
     <row r="281" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A281" s="1">
-        <v>16</v>
+        <v>60</v>
       </c>
       <c r="B281" s="2" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
     </row>
     <row r="282" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A282" s="1">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="B282" s="2" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
     </row>
     <row r="283" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A283" s="1">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="B283" s="2" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
     </row>
     <row r="284" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A284" s="1">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="B284" s="2" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="285" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A285" s="1">
-        <v>22</v>
-      </c>
-      <c r="B285" s="2" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="286" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A286" s="1">
-        <v>22</v>
-      </c>
-      <c r="B286" s="2" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="287" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A287" s="1">
-        <v>60</v>
-      </c>
-      <c r="B287" s="2" t="s">
         <v>277</v>
-      </c>
-    </row>
-    <row r="288" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A288" s="1">
-        <v>60</v>
-      </c>
-      <c r="B288" s="2" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="289" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A289" s="1">
-        <v>50</v>
-      </c>
-      <c r="B289" s="2" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="290" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A290" s="1">
-        <v>30</v>
-      </c>
-      <c r="B290" s="2" t="s">
-        <v>280</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add SUBRENT support for Section 8 rent rolls
</commit_message>
<xml_diff>
--- a/src/lib/automation/ie/reference/To add I&E.xlsx
+++ b/src/lib/automation/ie/reference/To add I&E.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8fcd883c776305f1/Documentos/Keystone/keystone-os/src/lib/automation/ie/reference/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="11_20C4315295263003D1BD0F964BC8F3756E9CBE04" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{043E67DD-55A6-48FC-B722-E28DA5DCE0F5}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="11_20C4315295263003D1BD0F964BC8F3756E9CBE04" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2F5D6694-CBDA-4896-9A44-23CD0AC90037}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3030" yWindow="2475" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -948,38 +948,12 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="3">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
-      </top>
-      <bottom style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
-      </right>
-      <top style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
-      </top>
-      <bottom style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -1009,54 +983,51 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1376,7 +1347,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:B284"/>
+  <dimension ref="A2:B281"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.28515625" customWidth="1"/>
@@ -2692,78 +2663,75 @@
       </c>
     </row>
     <row r="174" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A174" s="23">
+      <c r="A174" s="22">
         <v>42</v>
       </c>
-      <c r="B174" s="27" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
+      <c r="B174" s="14" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="175" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A175" s="22">
-        <v>42</v>
-      </c>
-      <c r="B175" s="14" t="s">
-        <v>170</v>
+      <c r="A175" s="23">
+        <v>11</v>
+      </c>
+      <c r="B175" s="17" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="176" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A176" s="23">
-        <v>11</v>
-      </c>
-      <c r="B176" s="17" t="s">
-        <v>171</v>
+      <c r="A176" s="22">
+        <v>11</v>
+      </c>
+      <c r="B176" s="14" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="177" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A177" s="22">
-        <v>11</v>
-      </c>
-      <c r="B177" s="14" t="s">
-        <v>172</v>
+      <c r="A177" s="1">
+        <v>110</v>
+      </c>
+      <c r="B177" s="2" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="178" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A178" s="22">
-        <v>41</v>
-      </c>
-      <c r="B178" s="30" t="str">
-        <f>B16</f>
-        <v>Other Income</v>
+      <c r="A178" s="1">
+        <v>110</v>
+      </c>
+      <c r="B178" s="2" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="179" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A179" s="31">
-        <v>42</v>
-      </c>
-      <c r="B179" s="32" t="str">
-        <f>B17</f>
-        <v>Insufficient Notice</v>
+      <c r="A179" s="1">
+        <v>120</v>
+      </c>
+      <c r="B179" s="2" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="180" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A180" s="1">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="B180" s="2" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
     </row>
     <row r="181" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A181" s="1">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="B181" s="2" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
     </row>
     <row r="182" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A182" s="1">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="B182" s="2" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
     </row>
     <row r="183" spans="1:2" x14ac:dyDescent="0.25">
@@ -2771,15 +2739,15 @@
         <v>115</v>
       </c>
       <c r="B183" s="2" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
     </row>
     <row r="184" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A184" s="1">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="B184" s="2" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
     </row>
     <row r="185" spans="1:2" x14ac:dyDescent="0.25">
@@ -2787,7 +2755,7 @@
         <v>115</v>
       </c>
       <c r="B185" s="2" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
     </row>
     <row r="186" spans="1:2" x14ac:dyDescent="0.25">
@@ -2795,7 +2763,7 @@
         <v>115</v>
       </c>
       <c r="B186" s="2" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
     </row>
     <row r="187" spans="1:2" x14ac:dyDescent="0.25">
@@ -2803,39 +2771,39 @@
         <v>121</v>
       </c>
       <c r="B187" s="2" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
     </row>
     <row r="188" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A188" s="1">
-        <v>115</v>
+        <v>142</v>
       </c>
       <c r="B188" s="2" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
     </row>
     <row r="189" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A189" s="1">
-        <v>115</v>
+        <v>160</v>
       </c>
       <c r="B189" s="2" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="190" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A190" s="1">
-        <v>121</v>
+        <v>140</v>
       </c>
       <c r="B190" s="2" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
     </row>
     <row r="191" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A191" s="1">
-        <v>142</v>
+        <v>160</v>
       </c>
       <c r="B191" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="192" spans="1:2" x14ac:dyDescent="0.25">
@@ -2843,23 +2811,23 @@
         <v>160</v>
       </c>
       <c r="B192" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
     </row>
     <row r="193" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A193" s="1">
-        <v>140</v>
+        <v>160</v>
       </c>
       <c r="B193" s="2" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
     </row>
     <row r="194" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A194" s="1">
-        <v>160</v>
+        <v>141</v>
       </c>
       <c r="B194" s="2" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
     </row>
     <row r="195" spans="1:2" x14ac:dyDescent="0.25">
@@ -2867,7 +2835,7 @@
         <v>160</v>
       </c>
       <c r="B195" s="2" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
     </row>
     <row r="196" spans="1:2" x14ac:dyDescent="0.25">
@@ -2875,15 +2843,15 @@
         <v>160</v>
       </c>
       <c r="B196" s="2" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
     </row>
     <row r="197" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A197" s="1">
-        <v>141</v>
+        <v>160</v>
       </c>
       <c r="B197" s="2" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
     </row>
     <row r="198" spans="1:2" x14ac:dyDescent="0.25">
@@ -2891,7 +2859,7 @@
         <v>160</v>
       </c>
       <c r="B198" s="2" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
     </row>
     <row r="199" spans="1:2" x14ac:dyDescent="0.25">
@@ -2899,7 +2867,7 @@
         <v>160</v>
       </c>
       <c r="B199" s="2" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
     </row>
     <row r="200" spans="1:2" x14ac:dyDescent="0.25">
@@ -2907,7 +2875,7 @@
         <v>160</v>
       </c>
       <c r="B200" s="2" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
     </row>
     <row r="201" spans="1:2" x14ac:dyDescent="0.25">
@@ -2915,7 +2883,7 @@
         <v>160</v>
       </c>
       <c r="B201" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
     </row>
     <row r="202" spans="1:2" x14ac:dyDescent="0.25">
@@ -2923,15 +2891,15 @@
         <v>160</v>
       </c>
       <c r="B202" s="2" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
     </row>
     <row r="203" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A203" s="1">
-        <v>160</v>
+        <v>103</v>
       </c>
       <c r="B203" s="2" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
     </row>
     <row r="204" spans="1:2" x14ac:dyDescent="0.25">
@@ -2939,15 +2907,15 @@
         <v>160</v>
       </c>
       <c r="B204" s="2" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
     </row>
     <row r="205" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A205" s="1">
-        <v>160</v>
+        <v>103</v>
       </c>
       <c r="B205" s="2" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
     </row>
     <row r="206" spans="1:2" x14ac:dyDescent="0.25">
@@ -2955,39 +2923,39 @@
         <v>103</v>
       </c>
       <c r="B206" s="2" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
     </row>
     <row r="207" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A207" s="1">
-        <v>160</v>
+        <v>103</v>
       </c>
       <c r="B207" s="2" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
     </row>
     <row r="208" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A208" s="1">
-        <v>103</v>
+        <v>41</v>
       </c>
       <c r="B208" s="2" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
     </row>
     <row r="209" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A209" s="1">
-        <v>103</v>
+        <v>41</v>
       </c>
       <c r="B209" s="2" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
     </row>
     <row r="210" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A210" s="1">
-        <v>103</v>
+        <v>41</v>
       </c>
       <c r="B210" s="2" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
     </row>
     <row r="211" spans="1:2" x14ac:dyDescent="0.25">
@@ -2995,7 +2963,7 @@
         <v>41</v>
       </c>
       <c r="B211" s="2" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
     </row>
     <row r="212" spans="1:2" x14ac:dyDescent="0.25">
@@ -3003,7 +2971,7 @@
         <v>41</v>
       </c>
       <c r="B212" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="213" spans="1:2" x14ac:dyDescent="0.25">
@@ -3011,7 +2979,7 @@
         <v>41</v>
       </c>
       <c r="B213" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
     </row>
     <row r="214" spans="1:2" x14ac:dyDescent="0.25">
@@ -3019,7 +2987,7 @@
         <v>41</v>
       </c>
       <c r="B214" s="2" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
     </row>
     <row r="215" spans="1:2" x14ac:dyDescent="0.25">
@@ -3027,7 +2995,7 @@
         <v>41</v>
       </c>
       <c r="B215" s="2" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
     </row>
     <row r="216" spans="1:2" x14ac:dyDescent="0.25">
@@ -3035,7 +3003,7 @@
         <v>41</v>
       </c>
       <c r="B216" s="2" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
     </row>
     <row r="217" spans="1:2" x14ac:dyDescent="0.25">
@@ -3043,7 +3011,7 @@
         <v>41</v>
       </c>
       <c r="B217" s="2" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
     </row>
     <row r="218" spans="1:2" x14ac:dyDescent="0.25">
@@ -3051,31 +3019,31 @@
         <v>41</v>
       </c>
       <c r="B218" s="2" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
     </row>
     <row r="219" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A219" s="1">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B219" s="2" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
     </row>
     <row r="220" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A220" s="1">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B220" s="2" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
     </row>
     <row r="221" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A221" s="1">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B221" s="2" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="222" spans="1:2" x14ac:dyDescent="0.25">
@@ -3083,7 +3051,7 @@
         <v>42</v>
       </c>
       <c r="B222" s="2" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="223" spans="1:2" x14ac:dyDescent="0.25">
@@ -3091,7 +3059,7 @@
         <v>42</v>
       </c>
       <c r="B223" s="2" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
     </row>
     <row r="224" spans="1:2" x14ac:dyDescent="0.25">
@@ -3099,7 +3067,7 @@
         <v>42</v>
       </c>
       <c r="B224" s="2" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
     </row>
     <row r="225" spans="1:2" x14ac:dyDescent="0.25">
@@ -3107,7 +3075,7 @@
         <v>42</v>
       </c>
       <c r="B225" s="2" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
     </row>
     <row r="226" spans="1:2" x14ac:dyDescent="0.25">
@@ -3115,7 +3083,7 @@
         <v>42</v>
       </c>
       <c r="B226" s="2" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
     </row>
     <row r="227" spans="1:2" x14ac:dyDescent="0.25">
@@ -3123,7 +3091,7 @@
         <v>42</v>
       </c>
       <c r="B227" s="2" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
     </row>
     <row r="228" spans="1:2" x14ac:dyDescent="0.25">
@@ -3131,31 +3099,31 @@
         <v>42</v>
       </c>
       <c r="B228" s="2" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
     </row>
     <row r="229" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A229" s="1">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B229" s="2" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
     </row>
     <row r="230" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A230" s="1">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B230" s="2" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
     </row>
     <row r="231" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A231" s="1">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B231" s="2" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
     </row>
     <row r="232" spans="1:2" x14ac:dyDescent="0.25">
@@ -3163,7 +3131,7 @@
         <v>43</v>
       </c>
       <c r="B232" s="2" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
     </row>
     <row r="233" spans="1:2" x14ac:dyDescent="0.25">
@@ -3171,7 +3139,7 @@
         <v>43</v>
       </c>
       <c r="B233" s="2" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
     </row>
     <row r="234" spans="1:2" x14ac:dyDescent="0.25">
@@ -3179,7 +3147,7 @@
         <v>43</v>
       </c>
       <c r="B234" s="2" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
     </row>
     <row r="235" spans="1:2" x14ac:dyDescent="0.25">
@@ -3187,7 +3155,7 @@
         <v>43</v>
       </c>
       <c r="B235" s="2" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
     </row>
     <row r="236" spans="1:2" x14ac:dyDescent="0.25">
@@ -3195,7 +3163,7 @@
         <v>43</v>
       </c>
       <c r="B236" s="2" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
     </row>
     <row r="237" spans="1:2" x14ac:dyDescent="0.25">
@@ -3203,7 +3171,7 @@
         <v>43</v>
       </c>
       <c r="B237" s="2" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
     </row>
     <row r="238" spans="1:2" x14ac:dyDescent="0.25">
@@ -3211,31 +3179,31 @@
         <v>43</v>
       </c>
       <c r="B238" s="2" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
     </row>
     <row r="239" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A239" s="1">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="B239" s="2" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
     </row>
     <row r="240" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A240" s="1">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="B240" s="2" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
     </row>
     <row r="241" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A241" s="1">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="B241" s="2" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
     </row>
     <row r="242" spans="1:2" x14ac:dyDescent="0.25">
@@ -3243,79 +3211,79 @@
         <v>12</v>
       </c>
       <c r="B242" s="2" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
     </row>
     <row r="243" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A243" s="1">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B243" s="2" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
     </row>
     <row r="244" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A244" s="1">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B244" s="2" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
     </row>
     <row r="245" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A245" s="1">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B245" s="2" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
     </row>
     <row r="246" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A246" s="1">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B246" s="2" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
     </row>
     <row r="247" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A247" s="1">
-        <v>11</v>
+        <v>41</v>
       </c>
       <c r="B247" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
     </row>
     <row r="248" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A248" s="1">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B248" s="2" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
     </row>
     <row r="249" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A249" s="1">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B249" s="2" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="250" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A250" s="1">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="B250" s="2" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
     </row>
     <row r="251" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A251" s="1">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B251" s="2" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
     </row>
     <row r="252" spans="1:2" x14ac:dyDescent="0.25">
@@ -3323,7 +3291,7 @@
         <v>11</v>
       </c>
       <c r="B252" s="2" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="253" spans="1:2" x14ac:dyDescent="0.25">
@@ -3331,7 +3299,7 @@
         <v>11</v>
       </c>
       <c r="B253" s="2" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
     </row>
     <row r="254" spans="1:2" x14ac:dyDescent="0.25">
@@ -3339,7 +3307,7 @@
         <v>11</v>
       </c>
       <c r="B254" s="2" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
     </row>
     <row r="255" spans="1:2" x14ac:dyDescent="0.25">
@@ -3347,7 +3315,7 @@
         <v>11</v>
       </c>
       <c r="B255" s="2" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
     </row>
     <row r="256" spans="1:2" x14ac:dyDescent="0.25">
@@ -3355,7 +3323,7 @@
         <v>11</v>
       </c>
       <c r="B256" s="2" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
     </row>
     <row r="257" spans="1:2" x14ac:dyDescent="0.25">
@@ -3363,7 +3331,7 @@
         <v>11</v>
       </c>
       <c r="B257" s="2" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="258" spans="1:2" x14ac:dyDescent="0.25">
@@ -3371,7 +3339,7 @@
         <v>11</v>
       </c>
       <c r="B258" s="2" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="259" spans="1:2" x14ac:dyDescent="0.25">
@@ -3379,7 +3347,7 @@
         <v>11</v>
       </c>
       <c r="B259" s="2" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="260" spans="1:2" x14ac:dyDescent="0.25">
@@ -3387,7 +3355,7 @@
         <v>11</v>
       </c>
       <c r="B260" s="2" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
     </row>
     <row r="261" spans="1:2" x14ac:dyDescent="0.25">
@@ -3395,15 +3363,15 @@
         <v>11</v>
       </c>
       <c r="B261" s="2" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
     </row>
     <row r="262" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A262" s="1">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B262" s="2" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
     </row>
     <row r="263" spans="1:2" x14ac:dyDescent="0.25">
@@ -3411,7 +3379,7 @@
         <v>11</v>
       </c>
       <c r="B263" s="2" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
     </row>
     <row r="264" spans="1:2" x14ac:dyDescent="0.25">
@@ -3419,15 +3387,15 @@
         <v>11</v>
       </c>
       <c r="B264" s="2" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
     </row>
     <row r="265" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A265" s="1">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B265" s="2" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
     </row>
     <row r="266" spans="1:2" x14ac:dyDescent="0.25">
@@ -3435,7 +3403,7 @@
         <v>11</v>
       </c>
       <c r="B266" s="2" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
     </row>
     <row r="267" spans="1:2" x14ac:dyDescent="0.25">
@@ -3443,7 +3411,7 @@
         <v>11</v>
       </c>
       <c r="B267" s="2" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
     </row>
     <row r="268" spans="1:2" x14ac:dyDescent="0.25">
@@ -3451,63 +3419,63 @@
         <v>11</v>
       </c>
       <c r="B268" s="2" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
     </row>
     <row r="269" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A269" s="1">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="B269" s="2" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
     </row>
     <row r="270" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A270" s="1">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="B270" s="2" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
     </row>
     <row r="271" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A271" s="1">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="B271" s="2" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
     </row>
     <row r="272" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A272" s="1">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="B272" s="2" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
     </row>
     <row r="273" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A273" s="1">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B273" s="2" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
     </row>
     <row r="274" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A274" s="1">
-        <v>22</v>
+        <v>41</v>
       </c>
       <c r="B274" s="2" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
     </row>
     <row r="275" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A275" s="1">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B275" s="2" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
     </row>
     <row r="276" spans="1:2" x14ac:dyDescent="0.25">
@@ -3515,70 +3483,46 @@
         <v>22</v>
       </c>
       <c r="B276" s="2" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
     </row>
     <row r="277" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A277" s="1">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="B277" s="2" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
     </row>
     <row r="278" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A278" s="1">
-        <v>21</v>
+        <v>60</v>
       </c>
       <c r="B278" s="2" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
     </row>
     <row r="279" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A279" s="1">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="B279" s="2" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
     </row>
     <row r="280" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A280" s="1">
-        <v>22</v>
+        <v>50</v>
       </c>
       <c r="B280" s="2" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
     </row>
     <row r="281" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A281" s="1">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="B281" s="2" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="282" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A282" s="1">
-        <v>60</v>
-      </c>
-      <c r="B282" s="2" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="283" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A283" s="1">
-        <v>50</v>
-      </c>
-      <c r="B283" s="2" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="284" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A284" s="1">
-        <v>30</v>
-      </c>
-      <c r="B284" s="2" t="s">
         <v>277</v>
       </c>
     </row>

</xml_diff>